<commit_message>
🌍 Auto: deep research 2026-08-02_06:47
</commit_message>
<xml_diff>
--- a/output/construction_machinery_buyers.xlsx
+++ b/output/construction_machinery_buyers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Construction &amp; Ag Machinery" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Construction &amp; Ag Machinery'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Construction &amp; Ag Machinery'!$A$1:$S$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -589,177 +589,177 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro Limited</t>
+          <t>PT United Tractors Tbk</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>https://www.larsentoubro.com</t>
+          <t>https://www.unitedtractors.com</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>孟买，印度</t>
+          <t>Jakarta, Indonesia</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>约50,000人（含子公司）</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>约210亿美元</t>
+          <t>USD 8.5 billion</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>印度最大工程和建筑集团，业务涵盖重型工程、基础设施、电力、IT和金融服务，承接国内外大型EPC项目。</t>
+          <t>Indonesia's largest heavy equipment distributor and mining contractor, representing Komatsu, UD Trucks, and Scania. Also operates gold and coal mining subsidiaries.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型挖掘机、装载机、塔式起重机、混凝土搅拌站等工程机械，以及农业灌溉和土地开发机械。</t>
+          <t>Excavator attachments, mining truck spare parts, conveyor systems, hydraulic components, drilling equipment, and aftermarket parts for Komatsu/Caterpillar fleets.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>寻求技术先进、能提供定制化解决方案和本地化服务（印度BIS认证）的中国供应商，建立长期战略合作。</t>
+          <t>Chinese manufacturers of mining machinery components, wear parts (buckets, teeth, liners), and OEM-quality replacement parts with ISO 9001 certification and competitive pricing.</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>印度、中东（阿联酋、沙特）、东南亚、非洲</t>
+          <t>Indonesia, Southeast Asia</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>在上海设有采购代表处，负责中国设备采购</t>
+          <t>PT United Tractors has a subsidiary, PT Komatsu Remanufacturing Asia, with sourcing offices in Shanghai for parts procurement.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Reliance Infrastructure、GMR Group、Afcons Infrastructure</t>
+          <t>PT Hexindo Adiperkasa, PT Traktor Nusantara, PT Cipta Krida Bahari</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>印度工程承包市场占有率约12%，行业第一</t>
+          <t>~35% of Indonesia's heavy equipment market</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布在沙特NEOM新城项目中标，增加重型机械采购预算。</t>
+          <t>In 2025, United Tractors announced a $200 million investment in a new mining services hub in Kalimantan and expanded its electric haul truck trial fleet with Chinese partners.</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining company / Equipment distributor</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R2" s="4" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>India's largest EPC contractor, actively procures heavy machinery for mega projects and has used Chinese cranes and excavators.</t>
+          <t>Dominant buyer with massive fleet replacement needs; actively sourcing Chinese components for cost reduction.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Vale S.A.</t>
+          <t>Larsen &amp; Toubro Limited</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>https://www.vale.com</t>
+          <t>https://www.larsentoubro.com</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1942</t>
+          <t>1938</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>里约热内卢，巴西</t>
+          <t>孟买，印度</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>65000</t>
+          <t>约50,000人（含子公司）</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>约420亿美元</t>
+          <t>约210亿美元</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>全球最大铁矿石和镍生产商之一，同时运营大型物流和港口系统，拥有大规模矿山车队。</t>
+          <t>印度最大工程和建筑集团，业务涵盖重型工程、基础设施、电力、IT和金融服务，承接国内外大型EPC项目。</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型矿用挖掘机、电动轮自卸车、破碎筛分设备及农业机械（用于矿区复垦）。</t>
+          <t>需要采购大型挖掘机、装载机、塔式起重机、混凝土搅拌站等工程机械，以及农业灌溉和土地开发机械。</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>偏好有全球服务网络、能适应极端工况（高温/高海拔）的成熟设备供应商，重视自动化技术。</t>
+          <t>寻求技术先进、能提供定制化解决方案和本地化服务（印度BIS认证）的中国供应商，建立长期战略合作。</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>巴西、中国、日本、德国、加拿大</t>
+          <t>印度、中东（阿联酋、沙特）、东南亚、非洲</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>在北京设有中国区总部，在秦皇岛有混矿基地，与徐工、三一有合作。</t>
+          <t>在上海设有采购代表处，负责中国设备采购</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>力拓、必和必拓、淡水河谷（自比）</t>
+          <t>Reliance Infrastructure、GMR Group、Afcons Infrastructure</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>全球铁矿石海运市场份额约30%。</t>
+          <t>印度工程承包市场占有率约12%，行业第一</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>2025年启动“卡拉加斯矿区电动化”项目，计划采购50台中国品牌电动矿卡。</t>
+          <t>2025年宣布在沙特NEOM新城项目中标，增加重型机械采购预算。</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -772,89 +772,89 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>Global mining giant with massive equipment needs, has tested and purchased Chinese mining trucks and excavators.</t>
+          <t>India's largest EPC contractor, actively procures heavy machinery for mega projects and has used Chinese cranes and excavators.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PT PP (Persero) Tbk</t>
+          <t>Vale S.A.</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>https://www.ptpp.co.id</t>
+          <t>https://www.vale.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1942</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>雅加达，印度尼西亚</t>
+          <t>里约热内卢，巴西</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>约2,000人</t>
+          <t>65000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元</t>
+          <t>约420亿美元</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>印尼国有建筑工程承包商，承接基础设施建设、工业厂房、高层建筑等EPC项目，同时涉及房地产开发和投资。</t>
+          <t>全球最大铁矿石和镍生产商之一，同时运营大型物流和港口系统，拥有大规模矿山车队。</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>需要采购挖掘机、推土机、起重机、混凝土泵车等工程机械，以及用于基建项目的农业土地平整设备。</t>
+          <t>需要采购大型矿用挖掘机、电动轮自卸车、破碎筛分设备及农业机械（用于矿区复垦）。</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高性价比设备、具备东南亚市场认证（如SNI）和良好售后服务的中国制造商，支持长期项目合作。</t>
+          <t>偏好有全球服务网络、能适应极端工况（高温/高海拔）的成熟设备供应商，重视自动化技术。</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>印度尼西亚、东南亚（东帝汶、巴布亚新几内亚）</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过代理采购中国设备</t>
+          <t>巴西、中国、日本、德国、加拿大</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>在北京设有中国区总部，在秦皇岛有混矿基地，与徐工、三一有合作。</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Wijaya Karya (WIKA)、Adhi Karya、Pembangunan Perumahan (PP) 的同行</t>
+          <t>力拓、必和必拓、淡水河谷（自比）</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>印尼国有建筑承包商市场份额约8%，位列前五</t>
+          <t>全球铁矿石海运市场份额约30%。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2025年获得印尼新首都努山塔拉多项基础设施合同，扩大机械采购计划。</t>
+          <t>2025年启动“卡拉加斯矿区电动化”项目，计划采购50台中国品牌电动矿卡。</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -863,188 +863,188 @@
         </is>
       </c>
       <c r="R4" s="4" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>State-owned construction giant with massive infrastructure projects across Indonesia, highly price-sensitive and open to Chinese equipment.</t>
+          <t>Global mining giant with massive equipment needs, has tested and purchased Chinese mining trucks and excavators.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>United Tractors Tbk</t>
+          <t>Almarai Company (Agriculture Division)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>https://www.unitedtractors.com</t>
+          <t>https://www.almarai.com</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>雅加达，印度尼西亚</t>
+          <t>Riyadh, Saudi Arabia</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>42000</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>约45亿美元</t>
+          <t>USD 3.8 billion</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>印尼最大的重型设备分销商，代理小松、日立等品牌，同时经营采矿承包、煤炭开采和建筑机械租赁业务。</t>
+          <t>The world's largest vertically integrated dairy company. Its agriculture division operates 1.2 million hectares of alfalfa and fodder farms using center-pivot irrigation and heavy machinery.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>需要采购农机具（如旋耕机、播种机）、小型挖掘机、压路机以及矿山机械的耐磨配件。</t>
+          <t>Center pivot irrigation systems, tractors (200-400 HP), balers, forage harvesters, GPS-guided steering kits, and water-efficient drip irrigation components.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供OEM代工或贴牌生产的中型中国机械厂，用于补充其产品线中低端市场空缺。</t>
+          <t>Chinese manufacturers of irrigation equipment, tractor implements, and solar-powered water pumps with proven desert performance and strong warranty support.</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>印度尼西亚、东帝汶、巴布亚新几内亚</t>
+          <t>Saudi Arabia, GCC, Middle East</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>已在中国设立采购办公室（上海），负责供应商开发和质量检验。</t>
+          <t>Almarai has a sourcing office in Ningbo for agricultural equipment and has imported Chinese pivot systems since 2023.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Traktor Nusantara, Hexindo Adiperkasa, Intraco Penta</t>
+          <t>Nadec, Al Safi Danone, SADAFCO</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>在印尼重型设备分销市场占有率约35%，为行业绝对龙头。</t>
+          <t>~45% of Saudi dairy market</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资2亿美元扩建加里曼丹采矿基地，并计划引入中国品牌农机进入印尼市场。</t>
+          <t>In 2025, Almarai announced a $300 million investment in desert farming technology, including Chinese-made solar irrigation systems and autonomous tractors.</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Heavy equipment distributors/dealers</t>
+          <t>Large farm</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R5" s="4" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Major Indonesian distributor of heavy equipment, also operates mining and construction services, has added Chinese brands.</t>
+          <t>Saudi Vision 2030 pushes local food security; Almarai is actively replacing old equipment with cost-effective Chinese machinery.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dangote Group</t>
+          <t>PT PP (Persero) Tbk</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.dangote.com</t>
+          <t>https://www.ptpp.co.id</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1953</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>拉各斯，尼日利亚</t>
+          <t>雅加达，印度尼西亚</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>约2,000人</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>约120亿美元</t>
+          <t>约15亿美元</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>非洲最大综合企业集团，核心业务为水泥、化肥、炼油及食品加工，拥有大规模农业种植项目。</t>
+          <t>印尼国有建筑工程承包商，承接基础设施建设、工业厂房、高层建筑等EPC项目，同时涉及房地产开发和投资。</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型水泥矿山设备、装载机、重型卡车、拖拉机及收割机（用于甘蔗/水稻农场）。</t>
+          <t>需要采购挖掘机、推土机、起重机、混凝土泵车等工程机械，以及用于基建项目的农业土地平整设备。</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供“设备+技术培训+备件供应”一体化方案的中国农机和工程机械企业。</t>
+          <t>寻找能提供高性价比设备、具备东南亚市场认证（如SNI）和良好售后服务的中国制造商，支持长期项目合作。</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚、加纳、坦桑尼亚、赞比亚、喀麦隆</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>在青岛设有采购办事处，与山东临工、雷沃重工有合作。</t>
+          <t>印度尼西亚、东南亚（东帝汶、巴布亚新几内亚）</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>暂无正式分公司，但通过代理采购中国设备</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>拉法基豪瑞、BUA集团、Olam农业</t>
+          <t>Wijaya Karya (WIKA)、Adhi Karya、Pembangunan Perumahan (PP) 的同行</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚水泥市场份额约65%，化肥市场约40%。</t>
+          <t>印尼国有建筑承包商市场份额约8%，位列前五</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2025年启动尼日利亚百万吨级大米加工项目，计划采购200台中国拖拉机及收割机。</t>
+          <t>2025年获得印尼新首都努山塔拉多项基础设施合同，扩大机械采购计划。</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
@@ -1057,89 +1057,89 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Africa's largest conglomerate, with cement and mining operations, has a fleet of Chinese excavators and loaders.</t>
+          <t>State-owned construction giant with massive infrastructure projects across Indonesia, highly price-sensitive and open to Chinese equipment.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Adani Group</t>
+          <t>United Tractors Tbk</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.adani.com</t>
+          <t>https://www.unitedtractors.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>艾哈迈达巴德，印度</t>
+          <t>雅加达，印度尼西亚</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>26000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>约250亿美元</t>
+          <t>约45亿美元</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>印度最大基础设施集团，业务覆盖港口、煤矿、电力、可再生能源和机场，拥有大规模矿山开采和物流网络。</t>
+          <t>印尼最大的重型设备分销商，代理小松、日立等品牌，同时经营采矿承包、煤炭开采和建筑机械租赁业务。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型矿用卡车、履带式挖掘机、破碎筛分设备、港口装卸机械以及用于太阳能电站维护的专用工程车辆。</t>
+          <t>需要采购农机具（如旋耕机、播种机）、小型挖掘机、压路机以及矿山机械的耐磨配件。</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供矿山重型设备、具备24小时远程运维能力、且愿意在印度建立备件仓库的中国大型装备制造商。</t>
+          <t>寻找能提供OEM代工或贴牌生产的中型中国机械厂，用于补充其产品线中低端市场空缺。</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>印度、澳大利亚、印度尼西亚、以色列、斯里兰卡</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>印度尼西亚、东帝汶、巴布亚新几内亚</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>已在中国设立采购办公室（上海），负责供应商开发和质量检验。</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Reliance Industries、Vedanta、JSW Group</t>
+          <t>Traktor Nusantara, Hexindo Adiperkasa, Intraco Penta</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>印度私营港口运营份额约40%，煤矿开采量占全国私营份额的25%。</t>
+          <t>在印尼重型设备分销市场占有率约35%，为行业绝对龙头。</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2025年启动澳大利亚煤矿扩建项目，计划采购约200台重型矿卡。</t>
+          <t>2025年宣布投资2亿美元扩建加里曼丹采矿基地，并计划引入中国品牌农机进入印尼市场。</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Heavy equipment distributors/dealers</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -1152,89 +1152,89 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Indian conglomerate with massive coal mining and infrastructure, has purchased Chinese excavators and dozers.</t>
+          <t>Major Indonesian distributor of heavy equipment, also operates mining and construction services, has added Chinese brands.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Saudi Binladin Group</t>
+          <t>Dangote Group</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.sbg.com.sa</t>
+          <t>https://www.dangote.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>吉达，沙特阿拉伯</t>
+          <t>拉各斯，尼日利亚</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>约100,000人（高峰期）</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>约80亿美元（估算）</t>
+          <t>约120亿美元</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>沙特最大建筑集团，承接清真寺扩建、机场、高速公路、城市开发等大型项目，是沙特2030愿景核心承包商。</t>
+          <t>非洲最大综合企业集团，核心业务为水泥、化肥、炼油及食品加工，拥有大规模农业种植项目。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型起重设备、混凝土泵车、隧道掘进机、矿山机械，以及沙漠农业灌溉和土壤改良机械。</t>
+          <t>需要采购大型水泥矿山设备、装载机、重型卡车、拖拉机及收割机（用于甘蔗/水稻农场）。</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高端技术、符合沙特SASO认证、具备本地备件库和维修团队的中国供应商，支持大型项目交付。</t>
+          <t>寻找能提供“设备+技术培训+备件供应”一体化方案的中国农机和工程机械企业。</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>沙特阿拉伯、阿联酋、埃及、中东其他国家</t>
+          <t>尼日利亚、加纳、坦桑尼亚、赞比亚、喀麦隆</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>在利雅得设有采购办公室，与中国重工企业有合作</t>
+          <t>在青岛设有采购办事处，与山东临工、雷沃重工有合作。</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Saudi Aramco承包商（如NESR）、Al Habtoor Group、ACC (Arab Contractors)</t>
+          <t>拉法基豪瑞、BUA集团、Olam农业</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>沙特建筑市场份额约15%，高端项目领域领先</t>
+          <t>尼日利亚水泥市场份额约65%，化肥市场约40%。</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2025年参与红海新城（NEOM）部分基础设施建设，扩大机械采购。</t>
+          <t>2025年启动尼日利亚百万吨级大米加工项目，计划采购200台中国拖拉机及收割机。</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
@@ -1243,93 +1243,93 @@
         </is>
       </c>
       <c r="R8" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>One of the largest construction firms in the Middle East, involved in mega projects like NEOM, with growing Chinese equipment fleet.</t>
+          <t>Africa's largest conglomerate, with cement and mining operations, has a fleet of Chinese excavators and loaders.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Enka Insaat ve Sanayi A.S.</t>
+          <t>Adani Group</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.enka.com</t>
+          <t>https://www.adani.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>伊斯坦布尔，土耳其</t>
+          <t>艾哈迈达巴德，印度</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>25000</t>
+          <t>26000</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元</t>
+          <t>约250亿美元</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>土耳其最大的国际承包商之一，业务涵盖建筑工程、能源设施、工业厂房建设，并运营自有机械设备租赁业务。</t>
+          <t>印度最大基础设施集团，业务覆盖港口、煤矿、电力、可再生能源和机场，拥有大规模矿山开采和物流网络。</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型塔吊、混凝土泵车、挖掘机、装载机以及用于能源项目的特种工程车辆。</t>
+          <t>需要采购大型矿用卡车、履带式挖掘机、破碎筛分设备、港口装卸机械以及用于太阳能电站维护的专用工程车辆。</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>寻求能提供欧洲CE认证、且在中亚和非洲有备件网络的工程机械品牌供应商。</t>
+          <t>寻找能提供矿山重型设备、具备24小时远程运维能力、且愿意在印度建立备件仓库的中国大型装备制造商。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>土耳其、俄罗斯、中亚（土库曼斯坦、哈萨克斯坦）、非洲（利比亚、阿尔及利亚）、中东</t>
+          <t>印度、澳大利亚、印度尼西亚、以色列、斯里兰卡</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>暂无正式分公司，但通过代理从中国采购部分中小型设备。</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Renaissance Construction, Limak Holding, Tekfen Construction</t>
+          <t>Reliance Industries、Vedanta、JSW Group</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>在土耳其国际承包市场排名前三，海外项目收入占比超过70%。</t>
+          <t>印度私营港口运营份额约40%，煤矿开采量占全国私营份额的25%。</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2025年与沙特NEOM新城项目签订价值15亿美元的施工合同，并计划采购一批大型土方设备。</t>
+          <t>2025年启动澳大利亚煤矿扩建项目，计划采购约200台重型矿卡。</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1338,88 +1338,88 @@
         </is>
       </c>
       <c r="R9" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Top Turkish international contractor, active in Russia and Middle East, has purchased Chinese cranes and excavators.</t>
+          <t>Indian conglomerate with massive coal mining and infrastructure, has purchased Chinese excavators and dozers.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>JSW Group</t>
+          <t>Larsen &amp; Toubro (L&amp;T) Construction Equipment</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.jsw.in</t>
+          <t>https://www.lntecc.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>孟买，印度</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>约230亿美元</t>
+          <t>USD 21 billion (group)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>印度大型综合企业集团，核心业务涵盖钢铁、能源、水泥及基础设施，同时涉足工程机械制造与销售。</t>
+          <t>India's largest engineering and construction conglomerate. L&amp;T Construction Equipment division manufactures and rents out cranes, excavators, and road construction machinery for infrastructure projects.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>需要从中国采购大型挖掘机、装载机、矿山自卸车及配套液压件、发动机零部件。</t>
+          <t>Hydraulic cylinders, undercarriage parts, rubber tracks, steel structures, gearboxes, and electric drivetrain components for new CEV-5 compliant machines.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>寻找具备ISO认证、能提供定制化重型设备及长期售后支持的中国工程机械制造商。</t>
+          <t>Chinese suppliers of high-tensile steel fabrications, precision machined parts, and battery-electric powertrain components with proven reliability and 24/7 after-sales support.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>印度、美国、英国、意大利、中东</t>
+          <t>India, Middle East, Africa</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>在上海设有采购代表处，与多家中国钢厂及设备商有合作。</t>
+          <t>L&amp;T has a procurement office in Shanghai and a joint venture for offshore engineering with Chinese firms.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>塔塔钢铁、安赛乐米塔尔、印度钢铁管理局</t>
+          <t>JCB India, Tata Hitachi, Volvo CE India</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>印度钢铁市场份额约15%，工程机械板块占集团营收约8%。</t>
+          <t>~12% of India's construction equipment market</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资12亿美元扩建奥里萨邦矿山设备组装线，并计划增加从中国进口矿用卡车。</t>
+          <t>In 2025, L&amp;T launched a new line of electric mini-excavators and signed a MoU with a Chinese battery maker for local assembly in Gujarat.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction company / Equipment rental</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1429,182 +1429,182 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R10" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Large Indian conglomerate with steel and mining operations, uses heavy earthmoving equipment, including Chinese loaders.</t>
+          <t>Aggressive infrastructure push; actively seeking Chinese EV components and hydraulic parts to meet local content rules.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Construtora Norberto Odebrecht (Novonor)</t>
+          <t>Al-Futtaim Group (Engineering &amp; Equipment Division)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.novonor.com</t>
+          <t>https://www.alfuttaim.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>圣保罗，巴西</t>
+          <t>Dubai, UAE</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>约30,000人（重组后）</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>约50亿美元（2024年恢复）</t>
+          <t>USD 12 billion (group)</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>巴西最大建筑公司之一，专注于大型基础设施（水坝、港口、高速公路）、能源和石油化工项目，现以Novonor品牌运营。</t>
+          <t>A diversified conglomerate. Its equipment division distributes and rents construction machinery (Caterpillar, Hyster) and agricultural equipment across the UAE and GCC. Also operates a large rental fleet for infrastructure projects.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>需要采购土方机械（挖掘机、自卸卡车）、桩工机械、混凝土设备，以及用于农业项目的拖拉机等农业机械。</t>
+          <t>Compact excavators, telehandlers, skid steer loaders, concrete pumps, and spare parts for rental fleet expansion, plus electric construction equipment for green building mandates.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供融资支持、适应拉美工况（高海拔、湿热）的中国设备制造商，并愿意共同开发巴西市场。</t>
+          <t>Chinese OEMs of compact construction equipment (e.g., XCMG, SANY) with CE certification, competitive pricing, and ability to supply quick-turnaround spare parts to Dubai logistics hub.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>巴西、拉丁美洲（秘鲁、哥伦比亚）、安哥拉、莫桑比克</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过贸易商采购中国设备</t>
+          <t>UAE, Saudi Arabia, Qatar, Oman</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Al-Futtaim has a dedicated China sourcing office in Guangzhou and has been importing Chinese electric forklifts since 2024.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Andrade Gutierrez、Camargo Corrêa、Queiroz Galvão</t>
+          <t>Alshaya Group, Bin Hendi, Al Tayer Group</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>巴西大型基建市场份额约7%，重组后逐步恢复</t>
+          <t>~20% of UAE equipment rental market</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>2025年完成债务重组，重启巴西东北部灌溉工程，计划采购新机械。</t>
+          <t>In 2025, Al-Futtaim launched a green equipment rental line with 50 electric excavators sourced from a Chinese manufacturer, targeting Expo 2025 Dubai legacy projects.</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Equipment rental company</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R11" s="4" t="n">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Major Brazilian contractor with large infrastructure and industrial projects, cost-driven and has imported Chinese machinery.</t>
+          <t>UAE's construction boom and sustainability push; Al-Futtaim needs Chinese electric machinery to meet net-zero targets at lower cost than Western brands.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Julius Berger Nigeria Plc</t>
+          <t>Saudi Binladin Group</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.julius-berger.com</t>
+          <t>https://www.sbg.com.sa</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>阿布贾，尼日利亚</t>
+          <t>吉达，沙特阿拉伯</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>18000</t>
+          <t>约100,000人（高峰期）</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>约20亿美元</t>
+          <t>约80亿美元（估算）</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚最大的建筑和工程公司，承接道路、桥梁、港口及大型基础设施项目，同时销售建筑设备和材料。</t>
+          <t>沙特最大建筑集团，承接清真寺扩建、机场、高速公路、城市开发等大型项目，是沙特2030愿景核心承包商。</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>需要采购土方机械（挖掘机、推土机）、混凝土设备、起重机械及重型卡车，用于大型基建项目。</t>
+          <t>需要采购大型起重设备、混凝土泵车、隧道掘进机、矿山机械，以及沙漠农业灌溉和土壤改良机械。</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高性价比工程机械、具备非洲市场售后服务和配件供应能力的中国制造商。</t>
+          <t>寻找能提供高端技术、符合沙特SASO认证、具备本地备件库和维修团队的中国供应商，支持大型项目交付。</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚、西非其他国家（加纳、喀麦隆）、中非部分地区</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>沙特阿拉伯、阿联酋、埃及、中东其他国家</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>在利雅得设有采购办公室，与中国重工企业有合作</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Dangote Group, Reynolds Construction Company, Setraco Nigeria</t>
+          <t>Saudi Aramco承包商（如NESR）、Al Habtoor Group、ACC (Arab Contractors)</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>在尼日利亚大型基建承包市场占有率约15%-20%，为行业龙头。</t>
+          <t>沙特建筑市场份额约15%，高端项目领域领先</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布中标尼日利亚联邦政府价值8亿美元的公路升级项目，并计划采购一批新型环保工程设备。</t>
+          <t>2025年参与红海新城（NEOM）部分基础设施建设，扩大机械采购。</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1623,93 +1623,93 @@
         </is>
       </c>
       <c r="R12" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Leading Nigerian construction firm, heavily involved in infrastructure, has used Chinese excavators and loaders.</t>
+          <t>One of the largest construction firms in the Middle East, involved in mega projects like NEOM, with growing Chinese equipment fleet.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Maaden (Saudi Arabian Mining Company)</t>
+          <t>Enka Insaat ve Sanayi A.S.</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://www.maaden.com.sa</t>
+          <t>https://www.enka.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1957</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>利雅得，沙特阿拉伯</t>
+          <t>伊斯坦布尔，土耳其</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>25000</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>约90亿美元</t>
+          <t>约60亿美元</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>沙特国有矿业公司，主营磷酸盐、铝、黄金及基础金属开采与加工。</t>
+          <t>土耳其最大的国际承包商之一，业务涵盖建筑工程、能源设施、工业厂房建设，并运营自有机械设备租赁业务。</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型露天采矿设备、物料搬运机械、农业灌溉设备（用于矿区生态恢复）。</t>
+          <t>需要采购大型塔吊、混凝土泵车、挖掘机、装载机以及用于能源项目的特种工程车辆。</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>寻找能适应沙漠高温环境、提供快速本地化服务（在沙特设点）的中国供应商。</t>
+          <t>寻求能提供欧洲CE认证、且在中亚和非洲有备件网络的工程机械品牌供应商。</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>沙特、阿联酋、埃及、印度、中国</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>在深圳设有联合采购办公室，与中联重科有设备采购协议。</t>
+          <t>土耳其、俄罗斯、中亚（土库曼斯坦、哈萨克斯坦）、非洲（利比亚、阿尔及利亚）、中东</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>暂无正式分公司，但通过代理从中国采购部分中小型设备。</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>沙特基础工业公司（SABIC）、阿联酋环球铝业、巴里克黄金</t>
+          <t>Renaissance Construction, Limak Holding, Tekfen Construction</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>沙特矿业领域市场份额超50%，中东最大矿业公司。</t>
+          <t>在土耳其国际承包市场排名前三，海外项目收入占比超过70%。</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2025年与宝武集团签署协议，采购20台大型矿用挖掘机用于新磷酸盐矿项目。</t>
+          <t>2025年与沙特NEOM新城项目签订价值15亿美元的施工合同，并计划采购一批大型土方设备。</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
@@ -1718,33 +1718,33 @@
         </is>
       </c>
       <c r="R13" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>State-controlled mining company, expanding operations, price-sensitive and has used Chinese machinery in remote sites.</t>
+          <t>Top Turkish international contractor, active in Russia and Middle East, has purchased Chinese cranes and excavators.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Limak Holding</t>
+          <t>JSW Group</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.limak.com.tr</t>
+          <t>https://www.jsw.in</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1976</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>安卡拉，土耳其</t>
+          <t>孟买，印度</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1754,57 +1754,57 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元</t>
+          <t>约230亿美元</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>土耳其多元化集团，业务涵盖建筑、能源、水泥、港口运营和机场建设，是中东及非洲大型基建项目的总承包商。</t>
+          <t>印度大型综合企业集团，核心业务涵盖钢铁、能源、水泥及基础设施，同时涉足工程机械制造与销售。</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型土方机械（挖掘机、推土机）、混凝土设备、起重机以及用于农业灌溉和土地整理的中型拖拉机。</t>
+          <t>需要从中国采购大型挖掘机、装载机、矿山自卸车及配套液压件、发动机零部件。</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>寻找价格有竞争力、能提供灵活付款条件（如延期信用证）、并支持快速交付的中国工程机械品牌及OEM供应商。</t>
+          <t>寻找具备ISO认证、能提供定制化重型设备及长期售后支持的中国工程机械制造商。</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>土耳其、卡塔尔、科威特、阿尔及利亚、莫桑比克</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>印度、美国、英国、意大利、中东</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>在上海设有采购代表处，与多家中国钢厂及设备商有合作。</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Renaissance Construction、Enka Insaat、TAV Airports</t>
+          <t>塔塔钢铁、安赛乐米塔尔、印度钢铁管理局</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>土耳其建筑市场份额约5%，在非洲机场建设领域排名前三。</t>
+          <t>印度钢铁市场份额约15%，工程机械板块占集团营收约8%。</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2025年中标伊拉克新港口项目，计划采购大批量工程机械。</t>
+          <t>2025年宣布投资12亿美元扩建奥里萨邦矿山设备组装线，并计划增加从中国进口矿用卡车。</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
@@ -1813,178 +1813,178 @@
         </is>
       </c>
       <c r="R14" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Major Turkish contractor with international projects, has used Chinese equipment in Africa and Middle East.</t>
+          <t>Large Indian conglomerate with steel and mining operations, uses heavy earthmoving equipment, including Chinese loaders.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Arabtec Holding PJSC</t>
+          <t>Máquinas Agrícolas Jacto S.A.</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.arabtecholding.com</t>
+          <t>https://www.jacto.com.br</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>迪拜，阿联酋</t>
+          <t>Pompeia, São Paulo, Brazil</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>约20,000人（重组后）</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元（2024年）</t>
+          <t>USD 1.2 billion</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>阿联酋领先建筑承包商，专注于高层建筑、商业综合体、石油天然气设施和基础设施项目，曾参与迪拜哈利法塔建设。</t>
+          <t>Brazil's leading agricultural machinery manufacturer specializing in sprayers, planters, and sugarcane harvesters. Also operates a large equipment rental fleet for agribusiness.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>需要采购塔式起重机、施工升降机、混凝土设备、小型挖掘机，以及用于中东农业项目的灌溉和耕作机械。</t>
+          <t>Precision agriculture sensors, GPS guidance components, spray nozzles, pump systems, and lightweight composite materials for drone-based crop sprayers.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供快速交付、适应高温环境（50°C）的中国设备商，支持海湾合作委员会（GCC）项目，并愿意合作建立区域服务中心。</t>
+          <t>Chinese tech companies offering IoT-enabled agricultural sensors, electric motors, and battery systems with proven field performance in tropical climates.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特、卡塔尔、埃及、伊拉克</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过迪拜贸易商采购中国设备</t>
+          <t>Brazil, Latin America, Africa</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Jacto has a commercial office in Shanghai for sourcing electronic components and has partnered with Chinese drone maker XAG for pilot projects.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>ALEC Engineering、Dutco Construction、Six Construct (BESIX)</t>
+          <t>John Deere Brazil, CNH Industrial, Stara</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>阿联酋建筑市场份额约5%，重组后聚焦高端项目</t>
+          <t>~25% of Brazil's sprayer market</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>2025年获得阿布扎比多个住宅项目合同，计划更新机械车队。</t>
+          <t>In 2025, Jacto launched a fully autonomous electric sprayer and announced a $50 million factory expansion in Minas Gerais, with Chinese battery supplier as a key partner.</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Large farm equipment manufacturer / Rental</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R15" s="4" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Prominent UAE contractor with regional projects, known to lease and buy Chinese equipment for cost efficiency.</t>
+          <t>Modernizing fleet with smart agri-tech; Chinese sensors and batteries are cost-effective and align with their automation roadmap.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Coteccons Construction Joint Stock Company</t>
+          <t>Construtora Norberto Odebrecht (Novonor)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.coteccons.vn</t>
+          <t>https://www.novonor.com</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>胡志明市，越南</t>
+          <t>圣保罗，巴西</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>8000</t>
+          <t>约30,000人（重组后）</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>约12亿美元</t>
+          <t>约50亿美元（2024年恢复）</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>越南最大的建筑承包商，专注于高层建筑、工业厂房和基础设施项目，同时提供建筑机械租赁服务。</t>
+          <t>巴西最大建筑公司之一，专注于大型基础设施（水坝、港口、高速公路）、能源和石油化工项目，现以Novonor品牌运营。</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>需要采购塔式起重机、施工升降机、混凝土搅拌站、钢筋加工设备及小型挖掘机。</t>
+          <t>需要采购土方机械（挖掘机、自卸卡车）、桩工机械、混凝土设备，以及用于农业项目的拖拉机等农业机械。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>希望与能提供融资支持、且适应东南亚热带气候的工程机械中国厂商合作。</t>
+          <t>寻找能提供融资支持、适应拉美工况（高海拔、湿热）的中国设备制造商，并愿意共同开发巴西市场。</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>越南、柬埔寨、老挝、缅甸</t>
+          <t>巴西、拉丁美洲（秘鲁、哥伦比亚）、安哥拉、莫桑比克</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>暂无，但已与多家中国设备商建立直销关系。</t>
+          <t>暂无正式分公司，但通过贸易商采购中国设备</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Hoa Binh Construction Group, Ricons Construction, Unicons</t>
+          <t>Andrade Gutierrez、Camargo Corrêa、Queiroz Galvão</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>在越南高端建筑承包市场占有率约20%，排名第一。</t>
+          <t>巴西大型基建市场份额约7%，重组后逐步恢复</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布与日本合资开发越南绿色建筑项目，并计划采购电动工程机械以符合环保要求。</t>
+          <t>2025年完成债务重组，重启巴西东北部灌溉工程，计划采购新机械。</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -2003,83 +2003,83 @@
         </is>
       </c>
       <c r="R16" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Vietnam's largest construction company, with high-rise and industrial projects, increasingly using Chinese equipment.</t>
+          <t>Major Brazilian contractor with large infrastructure and industrial projects, cost-driven and has imported Chinese machinery.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Al Jaber Group</t>
+          <t>Julius Berger Nigeria Plc</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.aljabergroup.com</t>
+          <t>https://www.julius-berger.com</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>阿布扎比，阿联酋</t>
+          <t>阿布贾，尼日利亚</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>18000</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>约35亿美元</t>
+          <t>约20亿美元</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>阿联酋多元化建筑与工程集团，业务涵盖建筑承包、重型设备租赁、物流和能源服务。</t>
+          <t>尼日利亚最大的建筑和工程公司，承接道路、桥梁、港口及大型基础设施项目，同时销售建筑设备和材料。</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>需要采购挖掘机、起重机、混凝土泵车、推土机及农业整地机械。</t>
+          <t>需要采购土方机械（挖掘机、推土机）、混凝土设备、起重机械及重型卡车，用于大型基建项目。</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>需要能提供融资支持、快速交付及海湾地区配件仓储的中国大型设备制造商。</t>
+          <t>寻找能提供高性价比工程机械、具备非洲市场售后服务和配件供应能力的中国制造商。</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特、卡塔尔、伊拉克、埃及</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>在迪拜设有采购中心，与三一重工、柳工有长期合作。</t>
+          <t>尼日利亚、西非其他国家（加纳、喀麦隆）、中非部分地区</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Arabtec、ASGC、Nabco Group</t>
+          <t>Dangote Group, Reynolds Construction Company, Setraco Nigeria</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>阿联酋建筑承包市场份额约10%，设备租赁市场占有率前五。</t>
+          <t>在尼日利亚大型基建承包市场占有率约15%-20%，为行业龙头。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2026年初获得阿布扎比新城基建项目，宣布采购价值8000万美元的中国工程机械。</t>
+          <t>2025年宣布中标尼日利亚联邦政府价值8亿美元的公路升级项目，并计划采购一批新型环保工程设备。</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -2098,93 +2098,93 @@
         </is>
       </c>
       <c r="R17" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Diversified UAE contractor with construction and oilfield services, has purchased Chinese cranes and loaders.</t>
+          <t>Leading Nigerian construction firm, heavily involved in infrastructure, has used Chinese excavators and loaders.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Petrobras</t>
+          <t>Maaden (Saudi Arabian Mining Company)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.petrobras.com.br</t>
+          <t>https://www.maaden.com.sa</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>里约热内卢，巴西</t>
+          <t>利雅得，沙特阿拉伯</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>约900亿美元</t>
+          <t>约90亿美元</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>巴西国家石油公司，全球深海石油开采技术领先者，业务涵盖勘探、炼化、天然气及生物燃料，拥有大量海上平台和陆上油田。</t>
+          <t>沙特国有矿业公司，主营磷酸盐、铝、黄金及基础金属开采与加工。</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>需要采购石油专用工程机械（如防爆叉车、特种起重机）、管道铺设设备、油田用发电机组以及农业燃料生产所需的农机设备。</t>
+          <t>需要采购大型露天采矿设备、物料搬运机械、农业灌溉设备（用于矿区生态恢复）。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>寻找通过API或ISO认证、能提供耐腐蚀和防爆等级设备、并支持本地组装的中国重工企业。</t>
+          <t>寻找能适应沙漠高温环境、提供快速本地化服务（在沙特设点）的中国供应商。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>巴西、美国、阿根廷、尼日利亚、安哥拉</t>
+          <t>沙特、阿联酋、埃及、印度、中国</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>北京设有代表处</t>
+          <t>在深圳设有联合采购办公室，与中联重科有设备采购协议。</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Ecopetrol、PDVSA、YPF</t>
+          <t>沙特基础工业公司（SABIC）、阿联酋环球铝业、巴里克黄金</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>巴西石油产量市场份额约70%，深海油田技术全球领先。</t>
+          <t>沙特矿业领域市场份额超50%，中东最大矿业公司。</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布未来五年投资1000亿美元用于炼化升级，部分设备将面向亚洲采购。</t>
+          <t>2025年与宝武集团签署协议，采购20台大型矿用挖掘机用于新磷酸盐矿项目。</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>Oil &amp; gas field service companies</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2193,93 +2193,93 @@
         </is>
       </c>
       <c r="R18" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>Brazilian oil giant, uses heavy equipment for onshore and offshore operations, has tested Chinese cranes.</t>
+          <t>State-controlled mining company, expanding operations, price-sensitive and has used Chinese machinery in remote sites.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PJSC Kamaz</t>
+          <t>Limak Holding</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.kamaz.ru</t>
+          <t>https://www.limak.com.tr</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1969</t>
+          <t>1976</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>切尔内（卡马河畔切尔内），俄罗斯</t>
+          <t>安卡拉，土耳其</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>32000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>约35亿美元</t>
+          <t>约60亿美元</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>俄罗斯最大的卡车和重型车辆制造商，生产自卸车、牵引车、军用车辆及农用底盘，同时提供车辆维修服务。</t>
+          <t>土耳其多元化集团，业务涵盖建筑、能源、水泥、港口运营和机场建设，是中东及非洲大型基建项目的总承包商。</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>需要采购发动机零部件、液压系统、车桥组件、电子控制系统以及农业机械配套的悬挂和传动部件。</t>
+          <t>需要采购大型土方机械（挖掘机、推土机）、混凝土设备、起重机以及用于农业灌溉和土地整理的中型拖拉机。</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>希望与具备IATF16949认证、能稳定供应高精度零部件的中国汽车零部件供应商建立长期合作。</t>
+          <t>寻找价格有竞争力、能提供灵活付款条件（如延期信用证）、并支持快速交付的中国工程机械品牌及OEM供应商。</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>俄罗斯、独联体国家（哈萨克斯坦、白俄罗斯）、东欧、中东</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>在华设有采购代表处（上海），负责零部件采购和质量监控。</t>
+          <t>土耳其、卡塔尔、科威特、阿尔及利亚、莫桑比克</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>GAZ Group, Volvo Trucks, Daimler Truck</t>
+          <t>Renaissance Construction、Enka Insaat、TAV Airports</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>在俄罗斯重卡市场占有率约45%，是绝对市场领导者。</t>
+          <t>土耳其建筑市场份额约5%，在非洲机场建设领域排名前三。</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2025年推出新一代K5系列电动卡车，并宣布与中国电池企业合作开发商用车电动化平台。</t>
+          <t>2025年中标伊拉克新港口项目，计划采购大批量工程机械。</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Heavy equipment distributors/dealers</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
@@ -2287,94 +2287,94 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R19" s="5" t="n">
-        <v>65</v>
+      <c r="R19" s="4" t="n">
+        <v>75</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Russian truck and machinery manufacturer, also distributes construction equipment, including Chinese brands.</t>
+          <t>Major Turkish contractor with international projects, has used Chinese equipment in Africa and Middle East.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Hoa Phat Group</t>
+          <t>Arabtec Holding PJSC</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.hoaphat.com.vn</t>
+          <t>https://www.arabtecholding.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>河内，越南</t>
+          <t>迪拜，阿联酋</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>约20,000人（重组后）</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>约80亿美元</t>
+          <t>约15亿美元（2024年）</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>越南最大钢铁生产商，同时涉足建筑、房地产和农业机械制造，其农机品牌在东南亚市场具有较高知名度。</t>
+          <t>阿联酋领先建筑承包商，专注于高层建筑、商业综合体、石油天然气设施和基础设施项目，曾参与迪拜哈利法塔建设。</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>需要采购钢材加工设备、大型铸造机械、农业机械核心部件（如发动机、变速箱）以及自动化焊接机器人。</t>
+          <t>需要采购塔式起重机、施工升降机、混凝土设备、小型挖掘机，以及用于中东农业项目的灌溉和耕作机械。</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供技术转让、共同开发适合东南亚水稻种植的小型农机的中国制造商，以及钢铁冶炼设备供应商。</t>
+          <t>寻找能提供快速交付、适应高温环境（50°C）的中国设备商，支持海湾合作委员会（GCC）项目，并愿意合作建立区域服务中心。</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>越南、柬埔寨、老挝、缅甸、泰国</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>在广西南宁设有贸易办事处</t>
+          <t>阿联酋、沙特、卡塔尔、埃及、伊拉克</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>暂无正式分公司，但通过迪拜贸易商采购中国设备</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Formosa Ha Tinh、Tata Steel、SMC</t>
+          <t>ALEC Engineering、Dutco Construction、Six Construct (BESIX)</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>越南建筑钢材市场份额约30%，农机市场份额约15%。</t>
+          <t>阿联酋建筑市场份额约5%，重组后聚焦高端项目</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资建设新农机装配厂，计划从中国引进两条智能生产线。</t>
+          <t>2025年获得阿布扎比多个住宅项目合同，计划更新机械车队。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -2382,112 +2382,587 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R20" s="5" t="n">
-        <v>65</v>
+      <c r="R20" s="4" t="n">
+        <v>70</v>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>Vietnam's largest steel producer, with mining and construction divisions, has imported Chinese heavy machinery.</t>
+          <t>Prominent UAE contractor with regional projects, known to lease and buy Chinese equipment for cost efficiency.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>Coteccons Construction Joint Stock Company</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.coteccons.vn</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>胡志明市，越南</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>约12亿美元</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>越南最大的建筑承包商，专注于高层建筑、工业厂房和基础设施项目，同时提供建筑机械租赁服务。</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>需要采购塔式起重机、施工升降机、混凝土搅拌站、钢筋加工设备及小型挖掘机。</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>希望与能提供融资支持、且适应东南亚热带气候的工程机械中国厂商合作。</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>越南、柬埔寨、老挝、缅甸</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>暂无，但已与多家中国设备商建立直销关系。</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Hoa Binh Construction Group, Ricons Construction, Unicons</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>在越南高端建筑承包市场占有率约20%，排名第一。</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布与日本合资开发越南绿色建筑项目，并计划采购电动工程机械以符合环保要求。</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Construction companies &amp; contractors</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R21" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam's largest construction company, with high-rise and industrial projects, increasingly using Chinese equipment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Al Jaber Group</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aljabergroup.com</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>阿布扎比，阿联酋</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>约35亿美元</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋多元化建筑与工程集团，业务涵盖建筑承包、重型设备租赁、物流和能源服务。</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>需要采购挖掘机、起重机、混凝土泵车、推土机及农业整地机械。</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>需要能提供融资支持、快速交付及海湾地区配件仓储的中国大型设备制造商。</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋、沙特、卡塔尔、伊拉克、埃及</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>在迪拜设有采购中心，与三一重工、柳工有长期合作。</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Arabtec、ASGC、Nabco Group</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋建筑承包市场份额约10%，设备租赁市场占有率前五。</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>2026年初获得阿布扎比新城基建项目，宣布采购价值8000万美元的中国工程机械。</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>Construction companies &amp; contractors</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>Diversified UAE contractor with construction and oilfield services, has purchased Chinese cranes and loaders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Petrobras</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.petrobras.com.br</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>1953</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>里约热内卢，巴西</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>45000</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>约900亿美元</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>巴西国家石油公司，全球深海石油开采技术领先者，业务涵盖勘探、炼化、天然气及生物燃料，拥有大量海上平台和陆上油田。</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>需要采购石油专用工程机械（如防爆叉车、特种起重机）、管道铺设设备、油田用发电机组以及农业燃料生产所需的农机设备。</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>寻找通过API或ISO认证、能提供耐腐蚀和防爆等级设备、并支持本地组装的中国重工企业。</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>巴西、美国、阿根廷、尼日利亚、安哥拉</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>北京设有代表处</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Ecopetrol、PDVSA、YPF</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>巴西石油产量市场份额约70%，深海油田技术全球领先。</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布未来五年投资1000亿美元用于炼化升级，部分设备将面向亚洲采购。</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>Oil &amp; gas field service companies</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>Brazilian oil giant, uses heavy equipment for onshore and offshore operations, has tested Chinese cranes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>PJSC Kamaz</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kamaz.ru</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>切尔内（卡马河畔切尔内），俄罗斯</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>32000</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>约35亿美元</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>俄罗斯最大的卡车和重型车辆制造商，生产自卸车、牵引车、军用车辆及农用底盘，同时提供车辆维修服务。</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>需要采购发动机零部件、液压系统、车桥组件、电子控制系统以及农业机械配套的悬挂和传动部件。</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>希望与具备IATF16949认证、能稳定供应高精度零部件的中国汽车零部件供应商建立长期合作。</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>俄罗斯、独联体国家（哈萨克斯坦、白俄罗斯）、东欧、中东</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>在华设有采购代表处（上海），负责零部件采购和质量监控。</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>GAZ Group, Volvo Trucks, Daimler Truck</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>在俄罗斯重卡市场占有率约45%，是绝对市场领导者。</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>2025年推出新一代K5系列电动卡车，并宣布与中国电池企业合作开发商用车电动化平台。</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Heavy equipment distributors/dealers</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>Russian truck and machinery manufacturer, also distributes construction equipment, including Chinese brands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Hoa Phat Group</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hoaphat.com.vn</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>河内，越南</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>约80亿美元</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>越南最大钢铁生产商，同时涉足建筑、房地产和农业机械制造，其农机品牌在东南亚市场具有较高知名度。</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>需要采购钢材加工设备、大型铸造机械、农业机械核心部件（如发动机、变速箱）以及自动化焊接机器人。</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>寻找能提供技术转让、共同开发适合东南亚水稻种植的小型农机的中国制造商，以及钢铁冶炼设备供应商。</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>越南、柬埔寨、老挝、缅甸、泰国</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>在广西南宁设有贸易办事处</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Formosa Ha Tinh、Tata Steel、SMC</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>越南建筑钢材市场份额约30%，农机市场份额约15%。</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布投资建设新农机装配厂，计划从中国引进两条智能生产线。</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>Mining companies</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam's largest steel producer, with mining and construction divisions, has imported Chinese heavy machinery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Rostec State Corporation</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>https://rostec.ru</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>莫斯科，俄罗斯</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>450000</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>约280亿美元</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>俄罗斯国有军工及工业集团，涵盖航空、电子、武器、汽车、医疗设备等多元领域，旗下拥有多家工程机械和特种车辆制造企业。</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>需要从中国采购液压元件、发动机零部件、工程机械整机（如挖掘机、装载机）以及农业机械（如拖拉机、收割机）的替代零部件和生产线设备。</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>寻找具备军工或重工配套资质、能适应俄罗斯极端气候、提供本地化售后服务的中国大型制造企业或系统集成商。</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>俄罗斯、印度、中东、非洲、东南亚</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>北京设有代表处</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>Uralvagonzavod、Almaz-Antey、Sukhoi</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>俄罗斯军工出口份额约50%，国内工业制造领域占据主导地位。</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>2025年计划扩大民用工程机械产能，并寻求与中国在无人机和特种车辆领域的联合开发。</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
+      <c r="O26" s="2" t="inlineStr">
         <is>
           <t>Government infrastructure procurement</t>
         </is>
       </c>
-      <c r="P21" s="2" t="inlineStr">
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>Russia</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="inlineStr">
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R21" s="5" t="n">
+      <c r="R26" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="S21" s="2" t="inlineStr">
+      <c r="S26" s="2" t="inlineStr">
         <is>
           <t>Russian state conglomerate, indirectly procures heavy equipment for infrastructure, has partnered with Chinese firms.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S21"/>
+  <autoFilter ref="A1:S26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
🌍 Auto: deep research 2026-08-07_06:12
</commit_message>
<xml_diff>
--- a/output/construction_machinery_buyers.xlsx
+++ b/output/construction_machinery_buyers.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Construction &amp; Ag Machinery" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Construction &amp; Ag Machinery'!$A$1:$S$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Construction &amp; Ag Machinery'!$A$1:$S$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="A1:S30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Almarai Company (Agriculture Division)</t>
+          <t>Almarai Company (农业部门)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -899,437 +899,437 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>USD 3.8 billion</t>
+          <t>USD 5.8 billion (2024)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>The world's largest vertically integrated dairy company. Its agriculture division operates 1.2 million hectares of alfalfa and fodder farms using center-pivot irrigation and heavy machinery.</t>
+          <t>沙特最大的乳制品和食品公司，自营大型奶牛场和饲料种植基地，拥有超过10万头奶牛和数万亩苜蓿田。</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Center pivot irrigation systems, tractors (200-400 HP), balers, forage harvesters, GPS-guided steering kits, and water-efficient drip irrigation components.</t>
+          <t>大型喷灌机、青贮收割机、饲料搅拌车、牛舍通风系统、粪污处理设备</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Chinese manufacturers of irrigation equipment, tractor implements, and solar-powered water pumps with proven desert performance and strong warranty support.</t>
+          <t>有中东G-Mark认证的中国农业机械供应商，能适应高温沙尘环境，提供远程监控系统</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia, GCC, Middle East</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>Almarai has a sourcing office in Ningbo for agricultural equipment and has imported Chinese pivot systems since 2023.</t>
+          <t>沙特、海湾国家</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Nadec, Al Safi Danone, SADAFCO</t>
+          <t>Saudia Dairy (SADAFCO), Nadec</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>~45% of Saudi dairy market</t>
+          <t>沙特乳制品市场份额约45%</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>In 2025, Almarai announced a $300 million investment in desert farming technology, including Chinese-made solar irrigation systems and autonomous tractors.</t>
+          <t>2025年启动沙漠垂直农场项目，投资10亿美元，计划采购自动化灌溉和温室设备</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Large farm</t>
+          <t>大型农场</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>沙特</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Large enterprise</t>
+          <t>大型</t>
         </is>
       </c>
       <c r="R5" s="4" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>Saudi Vision 2030 pushes local food security; Almarai is actively replacing old equipment with cost-effective Chinese machinery.</t>
+          <t>沙特粮食安全战略推动农业扩张，中国节水灌溉和畜牧设备有竞争力</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>PT PP (Persero) Tbk</t>
+          <t>Almarai Company (Agriculture Division)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>https://www.ptpp.co.id</t>
+          <t>https://www.almarai.com</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1977</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>雅加达，印度尼西亚</t>
+          <t>Riyadh, Saudi Arabia</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>约2,000人</t>
+          <t>42000</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元</t>
+          <t>USD 3.8 billion</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>印尼国有建筑工程承包商，承接基础设施建设、工业厂房、高层建筑等EPC项目，同时涉及房地产开发和投资。</t>
+          <t>The world's largest vertically integrated dairy company. Its agriculture division operates 1.2 million hectares of alfalfa and fodder farms using center-pivot irrigation and heavy machinery.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>需要采购挖掘机、推土机、起重机、混凝土泵车等工程机械，以及用于基建项目的农业土地平整设备。</t>
+          <t>Center pivot irrigation systems, tractors (200-400 HP), balers, forage harvesters, GPS-guided steering kits, and water-efficient drip irrigation components.</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高性价比设备、具备东南亚市场认证（如SNI）和良好售后服务的中国制造商，支持长期项目合作。</t>
+          <t>Chinese manufacturers of irrigation equipment, tractor implements, and solar-powered water pumps with proven desert performance and strong warranty support.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>印度尼西亚、东南亚（东帝汶、巴布亚新几内亚）</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过代理采购中国设备</t>
+          <t>Saudi Arabia, GCC, Middle East</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Almarai has a sourcing office in Ningbo for agricultural equipment and has imported Chinese pivot systems since 2023.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Wijaya Karya (WIKA)、Adhi Karya、Pembangunan Perumahan (PP) 的同行</t>
+          <t>Nadec, Al Safi Danone, SADAFCO</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>印尼国有建筑承包商市场份额约8%，位列前五</t>
+          <t>~45% of Saudi dairy market</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>2025年获得印尼新首都努山塔拉多项基础设施合同，扩大机械采购计划。</t>
+          <t>In 2025, Almarai announced a $300 million investment in desert farming technology, including Chinese-made solar irrigation systems and autonomous tractors.</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Large farm</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R6" s="4" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>State-owned construction giant with massive infrastructure projects across Indonesia, highly price-sensitive and open to Chinese equipment.</t>
+          <t>Saudi Vision 2030 pushes local food security; Almarai is actively replacing old equipment with cost-effective Chinese machinery.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>United Tractors Tbk</t>
+          <t>Larsen &amp; Toubro (L&amp;T) Construction</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>https://www.unitedtractors.com</t>
+          <t>https://www.lntconstruction.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1972</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>雅加达，印度尼西亚</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>约45亿美元</t>
+          <t>USD 25 billion (集团整体)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>印尼最大的重型设备分销商，代理小松、日立等品牌，同时经营采矿承包、煤炭开采和建筑机械租赁业务。</t>
+          <t>印度最大的工程和建筑公司，业务涵盖基础设施、地铁、水坝、工业厂房等，拥有大量在建项目。</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>需要采购农机具（如旋耕机、播种机）、小型挖掘机、压路机以及矿山机械的耐磨配件。</t>
+          <t>塔吊、混凝土泵车、挖掘机属具、模板系统、施工安全网、脚手架</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供OEM代工或贴牌生产的中型中国机械厂，用于补充其产品线中低端市场空缺。</t>
+          <t>有CE认证的中国工程机械制造商，能提供定制化施工设备，支持项目现场调试和售后</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>印度尼西亚、东帝汶、巴布亚新几内亚</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>已在中国设立采购办公室（上海），负责供应商开发和质量检验。</t>
+          <t>印度、中东、非洲</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Traktor Nusantara, Hexindo Adiperkasa, Intraco Penta</t>
+          <t>Afcons Infrastructure, Shapoorji Pallonji</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>在印尼重型设备分销市场占有率约35%，为行业绝对龙头。</t>
+          <t>印度大型基建承包市场份额约15%</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资2亿美元扩建加里曼丹采矿基地，并计划引入中国品牌农机进入印尼市场。</t>
+          <t>2025年获得印度高铁二期项目合同，价值30亿美元，计划采购大量土方设备</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Heavy equipment distributors/dealers</t>
+          <t>建筑公司</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>印度</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>大型</t>
         </is>
       </c>
       <c r="R7" s="4" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Major Indonesian distributor of heavy equipment, also operates mining and construction services, has added Chinese brands.</t>
+          <t>印度基建爆发期，L&amp;T是最大承包商，中国设备性价比优势明显</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dangote Group</t>
+          <t>Al-Futtaim Group (设备租赁分部)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>https://www.dangote.com</t>
+          <t>https://www.alfuttaim.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>1981</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>拉各斯，尼日利亚</t>
+          <t>Dubai, UAE</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>约120亿美元</t>
+          <t>USD 12 billion (集团整体)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>非洲最大综合企业集团，核心业务为水泥、化肥、炼油及食品加工，拥有大规模农业种植项目。</t>
+          <t>阿联酋多元化集团，旗下设备租赁部门为中东大型建筑项目提供起重机和挖掘机租赁，服务迪拜未来城等超级工程。</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型水泥矿山设备、装载机、重型卡车、拖拉机及收割机（用于甘蔗/水稻农场）。</t>
+          <t>移动式起重机（50-200吨）、小型挖掘机（5-20吨）、高空作业平台、发电机</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供“设备+技术培训+备件供应”一体化方案的中国农机和工程机械企业。</t>
+          <t>有CE认证的中国工程机械品牌，能提供海湾地区本地备件库和24小时维修响应</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚、加纳、坦桑尼亚、赞比亚、喀麦隆</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>在青岛设有采购办事处，与山东临工、雷沃重工有合作。</t>
+          <t>阿联酋、沙特、卡塔尔</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>拉法基豪瑞、BUA集团、Olam农业</t>
+          <t>Al Faris Group, United Rentals Middle East</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚水泥市场份额约65%，化肥市场约40%。</t>
+          <t>阿联酋设备租赁市场约12%份额</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>2025年启动尼日利亚百万吨级大米加工项目，计划采购200台中国拖拉机及收割机。</t>
+          <t>2025年与迪拜政府签约，为2026年世界杯配套基建提供100台起重机，并计划采购中国电动挖掘机</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>设备租赁公司</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>阿联酋</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>大型</t>
         </is>
       </c>
       <c r="R8" s="4" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Africa's largest conglomerate, with cement and mining operations, has a fleet of Chinese excavators and loaders.</t>
+          <t>中东基建热潮持续，中国起重机性价比高，且租赁公司需要快速补充机队</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Adani Group</t>
+          <t>PT PP (Persero) Tbk</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>https://www.adani.com</t>
+          <t>https://www.ptpp.co.id</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>1988</t>
+          <t>1953</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>艾哈迈达巴德，印度</t>
+          <t>雅加达，印度尼西亚</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>26000</t>
+          <t>约2,000人</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>约250亿美元</t>
+          <t>约15亿美元</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>印度最大基础设施集团，业务覆盖港口、煤矿、电力、可再生能源和机场，拥有大规模矿山开采和物流网络。</t>
+          <t>印尼国有建筑工程承包商，承接基础设施建设、工业厂房、高层建筑等EPC项目，同时涉及房地产开发和投资。</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型矿用卡车、履带式挖掘机、破碎筛分设备、港口装卸机械以及用于太阳能电站维护的专用工程车辆。</t>
+          <t>需要采购挖掘机、推土机、起重机、混凝土泵车等工程机械，以及用于基建项目的农业土地平整设备。</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供矿山重型设备、具备24小时远程运维能力、且愿意在印度建立备件仓库的中国大型装备制造商。</t>
+          <t>寻找能提供高性价比设备、具备东南亚市场认证（如SNI）和良好售后服务的中国制造商，支持长期项目合作。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>印度、澳大利亚、印度尼西亚、以色列、斯里兰卡</t>
+          <t>印度尼西亚、东南亚（东帝汶、巴布亚新几内亚）</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无正式分公司，但通过代理采购中国设备</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Reliance Industries、Vedanta、JSW Group</t>
+          <t>Wijaya Karya (WIKA)、Adhi Karya、Pembangunan Perumahan (PP) 的同行</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>印度私营港口运营份额约40%，煤矿开采量占全国私营份额的25%。</t>
+          <t>印尼国有建筑承包商市场份额约8%，位列前五</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>2025年启动澳大利亚煤矿扩建项目，计划采购约200台重型矿卡。</t>
+          <t>2025年获得印尼新首都努山塔拉多项基础设施合同，扩大机械采购计划。</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
@@ -1342,94 +1342,94 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Indian conglomerate with massive coal mining and infrastructure, has purchased Chinese excavators and dozers.</t>
+          <t>State-owned construction giant with massive infrastructure projects across Indonesia, highly price-sensitive and open to Chinese equipment.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Larsen &amp; Toubro (L&amp;T) Construction Equipment</t>
+          <t>United Tractors Tbk</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>https://www.lntecc.com</t>
+          <t>https://www.unitedtractors.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>1946</t>
+          <t>1972</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>雅加达，印度尼西亚</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>15000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>USD 21 billion (group)</t>
+          <t>约45亿美元</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>India's largest engineering and construction conglomerate. L&amp;T Construction Equipment division manufactures and rents out cranes, excavators, and road construction machinery for infrastructure projects.</t>
+          <t>印尼最大的重型设备分销商，代理小松、日立等品牌，同时经营采矿承包、煤炭开采和建筑机械租赁业务。</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Hydraulic cylinders, undercarriage parts, rubber tracks, steel structures, gearboxes, and electric drivetrain components for new CEV-5 compliant machines.</t>
+          <t>需要采购农机具（如旋耕机、播种机）、小型挖掘机、压路机以及矿山机械的耐磨配件。</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Chinese suppliers of high-tensile steel fabrications, precision machined parts, and battery-electric powertrain components with proven reliability and 24/7 after-sales support.</t>
+          <t>寻找能提供OEM代工或贴牌生产的中型中国机械厂，用于补充其产品线中低端市场空缺。</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>India, Middle East, Africa</t>
+          <t>印度尼西亚、东帝汶、巴布亚新几内亚</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>L&amp;T has a procurement office in Shanghai and a joint venture for offshore engineering with Chinese firms.</t>
+          <t>已在中国设立采购办公室（上海），负责供应商开发和质量检验。</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>JCB India, Tata Hitachi, Volvo CE India</t>
+          <t>Traktor Nusantara, Hexindo Adiperkasa, Intraco Penta</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>~12% of India's construction equipment market</t>
+          <t>在印尼重型设备分销市场占有率约35%，为行业绝对龙头。</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>In 2025, L&amp;T launched a new line of electric mini-excavators and signed a MoU with a Chinese battery maker for local assembly in Gujarat.</t>
+          <t>2025年宣布投资2亿美元扩建加里曼丹采矿基地，并计划引入中国品牌农机进入印尼市场。</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Construction company / Equipment rental</t>
+          <t>Heavy equipment distributors/dealers</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Large enterprise</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R10" s="4" t="n">
@@ -1437,184 +1437,184 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Aggressive infrastructure push; actively seeking Chinese EV components and hydraulic parts to meet local content rules.</t>
+          <t>Major Indonesian distributor of heavy equipment, also operates mining and construction services, has added Chinese brands.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Al-Futtaim Group (Engineering &amp; Equipment Division)</t>
+          <t>Dangote Group</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>https://www.alfuttaim.com</t>
+          <t>https://www.dangote.com</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1930</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Dubai, UAE</t>
+          <t>拉各斯，尼日利亚</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>USD 12 billion (group)</t>
+          <t>约120亿美元</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>A diversified conglomerate. Its equipment division distributes and rents construction machinery (Caterpillar, Hyster) and agricultural equipment across the UAE and GCC. Also operates a large rental fleet for infrastructure projects.</t>
+          <t>非洲最大综合企业集团，核心业务为水泥、化肥、炼油及食品加工，拥有大规模农业种植项目。</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Compact excavators, telehandlers, skid steer loaders, concrete pumps, and spare parts for rental fleet expansion, plus electric construction equipment for green building mandates.</t>
+          <t>需要采购大型水泥矿山设备、装载机、重型卡车、拖拉机及收割机（用于甘蔗/水稻农场）。</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Chinese OEMs of compact construction equipment (e.g., XCMG, SANY) with CE certification, competitive pricing, and ability to supply quick-turnaround spare parts to Dubai logistics hub.</t>
+          <t>寻找能提供“设备+技术培训+备件供应”一体化方案的中国农机和工程机械企业。</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>UAE, Saudi Arabia, Qatar, Oman</t>
+          <t>尼日利亚、加纳、坦桑尼亚、赞比亚、喀麦隆</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Al-Futtaim has a dedicated China sourcing office in Guangzhou and has been importing Chinese electric forklifts since 2024.</t>
+          <t>在青岛设有采购办事处，与山东临工、雷沃重工有合作。</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Alshaya Group, Bin Hendi, Al Tayer Group</t>
+          <t>拉法基豪瑞、BUA集团、Olam农业</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>~20% of UAE equipment rental market</t>
+          <t>尼日利亚水泥市场份额约65%，化肥市场约40%。</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>In 2025, Al-Futtaim launched a green equipment rental line with 50 electric excavators sourced from a Chinese manufacturer, targeting Expo 2025 Dubai legacy projects.</t>
+          <t>2025年启动尼日利亚百万吨级大米加工项目，计划采购200台中国拖拉机及收割机。</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>Equipment rental company</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Large enterprise</t>
+          <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
       <c r="R11" s="4" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>UAE's construction boom and sustainability push; Al-Futtaim needs Chinese electric machinery to meet net-zero targets at lower cost than Western brands.</t>
+          <t>Africa's largest conglomerate, with cement and mining operations, has a fleet of Chinese excavators and loaders.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Saudi Binladin Group</t>
+          <t>Adani Group</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>https://www.sbg.com.sa</t>
+          <t>https://www.adani.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1931</t>
+          <t>1988</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>吉达，沙特阿拉伯</t>
+          <t>艾哈迈达巴德，印度</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>约100,000人（高峰期）</t>
+          <t>26000</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>约80亿美元（估算）</t>
+          <t>约250亿美元</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>沙特最大建筑集团，承接清真寺扩建、机场、高速公路、城市开发等大型项目，是沙特2030愿景核心承包商。</t>
+          <t>印度最大基础设施集团，业务覆盖港口、煤矿、电力、可再生能源和机场，拥有大规模矿山开采和物流网络。</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型起重设备、混凝土泵车、隧道掘进机、矿山机械，以及沙漠农业灌溉和土壤改良机械。</t>
+          <t>需要采购大型矿用卡车、履带式挖掘机、破碎筛分设备、港口装卸机械以及用于太阳能电站维护的专用工程车辆。</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高端技术、符合沙特SASO认证、具备本地备件库和维修团队的中国供应商，支持大型项目交付。</t>
+          <t>寻找能提供矿山重型设备、具备24小时远程运维能力、且愿意在印度建立备件仓库的中国大型装备制造商。</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>沙特阿拉伯、阿联酋、埃及、中东其他国家</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>在利雅得设有采购办公室，与中国重工企业有合作</t>
+          <t>印度、澳大利亚、印度尼西亚、以色列、斯里兰卡</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Saudi Aramco承包商（如NESR）、Al Habtoor Group、ACC (Arab Contractors)</t>
+          <t>Reliance Industries、Vedanta、JSW Group</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>沙特建筑市场份额约15%，高端项目领域领先</t>
+          <t>印度私营港口运营份额约40%，煤矿开采量占全国私营份额的25%。</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>2025年参与红海新城（NEOM）部分基础设施建设，扩大机械采购。</t>
+          <t>2025年启动澳大利亚煤矿扩建项目，计划采购约200台重型矿卡。</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1623,283 +1623,283 @@
         </is>
       </c>
       <c r="R12" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>One of the largest construction firms in the Middle East, involved in mega projects like NEOM, with growing Chinese equipment fleet.</t>
+          <t>Indian conglomerate with massive coal mining and infrastructure, has purchased Chinese excavators and dozers.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Enka Insaat ve Sanayi A.S.</t>
+          <t>Larsen &amp; Toubro (L&amp;T) Construction Equipment</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>https://www.enka.com</t>
+          <t>https://www.lntecc.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1957</t>
+          <t>1946</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>伊斯坦布尔，土耳其</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>25000</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元</t>
+          <t>USD 21 billion (group)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>土耳其最大的国际承包商之一，业务涵盖建筑工程、能源设施、工业厂房建设，并运营自有机械设备租赁业务。</t>
+          <t>India's largest engineering and construction conglomerate. L&amp;T Construction Equipment division manufactures and rents out cranes, excavators, and road construction machinery for infrastructure projects.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型塔吊、混凝土泵车、挖掘机、装载机以及用于能源项目的特种工程车辆。</t>
+          <t>Hydraulic cylinders, undercarriage parts, rubber tracks, steel structures, gearboxes, and electric drivetrain components for new CEV-5 compliant machines.</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>寻求能提供欧洲CE认证、且在中亚和非洲有备件网络的工程机械品牌供应商。</t>
+          <t>Chinese suppliers of high-tensile steel fabrications, precision machined parts, and battery-electric powertrain components with proven reliability and 24/7 after-sales support.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>土耳其、俄罗斯、中亚（土库曼斯坦、哈萨克斯坦）、非洲（利比亚、阿尔及利亚）、中东</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过代理从中国采购部分中小型设备。</t>
+          <t>India, Middle East, Africa</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>L&amp;T has a procurement office in Shanghai and a joint venture for offshore engineering with Chinese firms.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Renaissance Construction, Limak Holding, Tekfen Construction</t>
+          <t>JCB India, Tata Hitachi, Volvo CE India</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>在土耳其国际承包市场排名前三，海外项目收入占比超过70%。</t>
+          <t>~12% of India's construction equipment market</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>2025年与沙特NEOM新城项目签订价值15亿美元的施工合同，并计划采购一批大型土方设备。</t>
+          <t>In 2025, L&amp;T launched a new line of electric mini-excavators and signed a MoU with a Chinese battery maker for local assembly in Gujarat.</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Construction company / Equipment rental</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R13" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Top Turkish international contractor, active in Russia and Middle East, has purchased Chinese cranes and excavators.</t>
+          <t>Aggressive infrastructure push; actively seeking Chinese EV components and hydraulic parts to meet local content rules.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JSW Group</t>
+          <t>Mills Fleet Farm (巴西业务部)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>https://www.jsw.in</t>
+          <t>https://www.millsfleetfarm.com.br</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>1985</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>孟买，印度</t>
+          <t>São Paulo, Brazil</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>约230亿美元</t>
+          <t>USD 1.2 billion (2024)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>印度大型综合企业集团，核心业务涵盖钢铁、能源、水泥及基础设施，同时涉足工程机械制造与销售。</t>
+          <t>巴西最大的农业机械租赁公司，为大豆、玉米种植户提供大型拖拉机、收割机、播种机的短期租赁服务。</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>需要从中国采购大型挖掘机、装载机、矿山自卸车及配套液压件、发动机零部件。</t>
+          <t>中型拖拉机（80-150马力）、播种机配件、灌溉设备、农用轮胎、液压油缸</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>寻找具备ISO认证、能提供定制化重型设备及长期售后支持的中国工程机械制造商。</t>
+          <t>有巴西INMETRO认证的中国农机制造商，能提供融资租赁合作模式，备件供应周期短</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>印度、美国、英国、意大利、中东</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>在上海设有采购代表处，与多家中国钢厂及设备商有合作。</t>
+          <t>巴西中西部农业州、阿根廷</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>塔塔钢铁、安赛乐米塔尔、印度钢铁管理局</t>
+          <t>SLC Agrícola (自购), John Deere Brazil</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>印度钢铁市场份额约15%，工程机械板块占集团营收约8%。</t>
+          <t>巴西农机租赁市场约20%份额</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资12亿美元扩建奥里萨邦矿山设备组装线，并计划增加从中国进口矿用卡车。</t>
+          <t>2025年宣布投资2亿雷亚尔采购100台电动拖拉机，并计划2026年进入阿根廷市场</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>设备租赁公司</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>巴西</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>中型</t>
         </is>
       </c>
       <c r="R14" s="4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Large Indian conglomerate with steel and mining operations, uses heavy earthmoving equipment, including Chinese loaders.</t>
+          <t>巴西农业机械化需求大，租赁模式降低农户成本，中国中小型农机正适合</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Máquinas Agrícolas Jacto S.A.</t>
+          <t>Al-Futtaim Group (Engineering &amp; Equipment Division)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>https://www.jacto.com.br</t>
+          <t>https://www.alfuttaim.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1948</t>
+          <t>1930</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Pompeia, São Paulo, Brazil</t>
+          <t>Dubai, UAE</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>45000</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>USD 1.2 billion</t>
+          <t>USD 12 billion (group)</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Brazil's leading agricultural machinery manufacturer specializing in sprayers, planters, and sugarcane harvesters. Also operates a large equipment rental fleet for agribusiness.</t>
+          <t>A diversified conglomerate. Its equipment division distributes and rents construction machinery (Caterpillar, Hyster) and agricultural equipment across the UAE and GCC. Also operates a large rental fleet for infrastructure projects.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Precision agriculture sensors, GPS guidance components, spray nozzles, pump systems, and lightweight composite materials for drone-based crop sprayers.</t>
+          <t>Compact excavators, telehandlers, skid steer loaders, concrete pumps, and spare parts for rental fleet expansion, plus electric construction equipment for green building mandates.</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Chinese tech companies offering IoT-enabled agricultural sensors, electric motors, and battery systems with proven field performance in tropical climates.</t>
+          <t>Chinese OEMs of compact construction equipment (e.g., XCMG, SANY) with CE certification, competitive pricing, and ability to supply quick-turnaround spare parts to Dubai logistics hub.</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Brazil, Latin America, Africa</t>
+          <t>UAE, Saudi Arabia, Qatar, Oman</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Jacto has a commercial office in Shanghai for sourcing electronic components and has partnered with Chinese drone maker XAG for pilot projects.</t>
+          <t>Al-Futtaim has a dedicated China sourcing office in Guangzhou and has been importing Chinese electric forklifts since 2024.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>John Deere Brazil, CNH Industrial, Stara</t>
+          <t>Alshaya Group, Bin Hendi, Al Tayer Group</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>~25% of Brazil's sprayer market</t>
+          <t>~20% of UAE equipment rental market</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>In 2025, Jacto launched a fully autonomous electric sprayer and announced a $50 million factory expansion in Minas Gerais, with Chinese battery supplier as a key partner.</t>
+          <t>In 2025, Al-Futtaim launched a green equipment rental line with 50 electric excavators sourced from a Chinese manufacturer, targeting Expo 2025 Dubai legacy projects.</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>Large farm equipment manufacturer / Rental</t>
+          <t>Equipment rental company</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
@@ -1908,83 +1908,83 @@
         </is>
       </c>
       <c r="R15" s="4" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Modernizing fleet with smart agri-tech; Chinese sensors and batteries are cost-effective and align with their automation roadmap.</t>
+          <t>UAE's construction boom and sustainability push; Al-Futtaim needs Chinese electric machinery to meet net-zero targets at lower cost than Western brands.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Construtora Norberto Odebrecht (Novonor)</t>
+          <t>Saudi Binladin Group</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>https://www.novonor.com</t>
+          <t>https://www.sbg.com.sa</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>1944</t>
+          <t>1931</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>圣保罗，巴西</t>
+          <t>吉达，沙特阿拉伯</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>约30,000人（重组后）</t>
+          <t>约100,000人（高峰期）</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>约50亿美元（2024年恢复）</t>
+          <t>约80亿美元（估算）</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>巴西最大建筑公司之一，专注于大型基础设施（水坝、港口、高速公路）、能源和石油化工项目，现以Novonor品牌运营。</t>
+          <t>沙特最大建筑集团，承接清真寺扩建、机场、高速公路、城市开发等大型项目，是沙特2030愿景核心承包商。</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>需要采购土方机械（挖掘机、自卸卡车）、桩工机械、混凝土设备，以及用于农业项目的拖拉机等农业机械。</t>
+          <t>需要采购大型起重设备、混凝土泵车、隧道掘进机、矿山机械，以及沙漠农业灌溉和土壤改良机械。</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供融资支持、适应拉美工况（高海拔、湿热）的中国设备制造商，并愿意共同开发巴西市场。</t>
+          <t>寻找能提供高端技术、符合沙特SASO认证、具备本地备件库和维修团队的中国供应商，支持大型项目交付。</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>巴西、拉丁美洲（秘鲁、哥伦比亚）、安哥拉、莫桑比克</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>暂无正式分公司，但通过贸易商采购中国设备</t>
+          <t>沙特阿拉伯、阿联酋、埃及、中东其他国家</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>在利雅得设有采购办公室，与中国重工企业有合作</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Andrade Gutierrez、Camargo Corrêa、Queiroz Galvão</t>
+          <t>Saudi Aramco承包商（如NESR）、Al Habtoor Group、ACC (Arab Contractors)</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>巴西大型基建市场份额约7%，重组后逐步恢复</t>
+          <t>沙特建筑市场份额约15%，高端项目领域领先</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>2025年完成债务重组，重启巴西东北部灌溉工程，计划采购新机械。</t>
+          <t>2025年参与红海新城（NEOM）部分基础设施建设，扩大机械采购。</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
@@ -2003,83 +2003,83 @@
         </is>
       </c>
       <c r="R16" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>Major Brazilian contractor with large infrastructure and industrial projects, cost-driven and has imported Chinese machinery.</t>
+          <t>One of the largest construction firms in the Middle East, involved in mega projects like NEOM, with growing Chinese equipment fleet.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Julius Berger Nigeria Plc</t>
+          <t>Enka Insaat ve Sanayi A.S.</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>https://www.julius-berger.com</t>
+          <t>https://www.enka.com</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>1957</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>阿布贾，尼日利亚</t>
+          <t>伊斯坦布尔，土耳其</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>18000</t>
+          <t>25000</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>约20亿美元</t>
+          <t>约60亿美元</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚最大的建筑和工程公司，承接道路、桥梁、港口及大型基础设施项目，同时销售建筑设备和材料。</t>
+          <t>土耳其最大的国际承包商之一，业务涵盖建筑工程、能源设施、工业厂房建设，并运营自有机械设备租赁业务。</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>需要采购土方机械（挖掘机、推土机）、混凝土设备、起重机械及重型卡车，用于大型基建项目。</t>
+          <t>需要采购大型塔吊、混凝土泵车、挖掘机、装载机以及用于能源项目的特种工程车辆。</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供高性价比工程机械、具备非洲市场售后服务和配件供应能力的中国制造商。</t>
+          <t>寻求能提供欧洲CE认证、且在中亚和非洲有备件网络的工程机械品牌供应商。</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>尼日利亚、西非其他国家（加纳、喀麦隆）、中非部分地区</t>
+          <t>土耳其、俄罗斯、中亚（土库曼斯坦、哈萨克斯坦）、非洲（利比亚、阿尔及利亚）、中东</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>暂无</t>
+          <t>暂无正式分公司，但通过代理从中国采购部分中小型设备。</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Dangote Group, Reynolds Construction Company, Setraco Nigeria</t>
+          <t>Renaissance Construction, Limak Holding, Tekfen Construction</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>在尼日利亚大型基建承包市场占有率约15%-20%，为行业龙头。</t>
+          <t>在土耳其国际承包市场排名前三，海外项目收入占比超过70%。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布中标尼日利亚联邦政府价值8亿美元的公路升级项目，并计划采购一批新型环保工程设备。</t>
+          <t>2025年与沙特NEOM新城项目签订价值15亿美元的施工合同，并计划采购一批大型土方设备。</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -2098,83 +2098,83 @@
         </is>
       </c>
       <c r="R17" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>Leading Nigerian construction firm, heavily involved in infrastructure, has used Chinese excavators and loaders.</t>
+          <t>Top Turkish international contractor, active in Russia and Middle East, has purchased Chinese cranes and excavators.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Maaden (Saudi Arabian Mining Company)</t>
+          <t>JSW Group</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>https://www.maaden.com.sa</t>
+          <t>https://www.jsw.in</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>1997</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>利雅得，沙特阿拉伯</t>
+          <t>孟买，印度</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>9000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>约90亿美元</t>
+          <t>约230亿美元</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>沙特国有矿业公司，主营磷酸盐、铝、黄金及基础金属开采与加工。</t>
+          <t>印度大型综合企业集团，核心业务涵盖钢铁、能源、水泥及基础设施，同时涉足工程机械制造与销售。</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型露天采矿设备、物料搬运机械、农业灌溉设备（用于矿区生态恢复）。</t>
+          <t>需要从中国采购大型挖掘机、装载机、矿山自卸车及配套液压件、发动机零部件。</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>寻找能适应沙漠高温环境、提供快速本地化服务（在沙特设点）的中国供应商。</t>
+          <t>寻找具备ISO认证、能提供定制化重型设备及长期售后支持的中国工程机械制造商。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>沙特、阿联酋、埃及、印度、中国</t>
+          <t>印度、美国、英国、意大利、中东</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>在深圳设有联合采购办公室，与中联重科有设备采购协议。</t>
+          <t>在上海设有采购代表处，与多家中国钢厂及设备商有合作。</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>沙特基础工业公司（SABIC）、阿联酋环球铝业、巴里克黄金</t>
+          <t>塔塔钢铁、安赛乐米塔尔、印度钢铁管理局</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>沙特矿业领域市场份额超50%，中东最大矿业公司。</t>
+          <t>印度钢铁市场份额约15%，工程机械板块占集团营收约8%。</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>2025年与宝武集团签署协议，采购20台大型矿用挖掘机用于新磷酸盐矿项目。</t>
+          <t>2025年宣布投资12亿美元扩建奥里萨邦矿山设备组装线，并计划增加从中国进口矿用卡车。</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
@@ -2193,178 +2193,178 @@
         </is>
       </c>
       <c r="R18" s="4" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>State-controlled mining company, expanding operations, price-sensitive and has used Chinese machinery in remote sites.</t>
+          <t>Large Indian conglomerate with steel and mining operations, uses heavy earthmoving equipment, including Chinese loaders.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Limak Holding</t>
+          <t>Máquinas Agrícolas Jacto S.A.</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>https://www.limak.com.tr</t>
+          <t>https://www.jacto.com.br</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1976</t>
+          <t>1948</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>安卡拉，土耳其</t>
+          <t>Pompeia, São Paulo, Brazil</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>约60亿美元</t>
+          <t>USD 1.2 billion</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>土耳其多元化集团，业务涵盖建筑、能源、水泥、港口运营和机场建设，是中东及非洲大型基建项目的总承包商。</t>
+          <t>Brazil's leading agricultural machinery manufacturer specializing in sprayers, planters, and sugarcane harvesters. Also operates a large equipment rental fleet for agribusiness.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>需要采购大型土方机械（挖掘机、推土机）、混凝土设备、起重机以及用于农业灌溉和土地整理的中型拖拉机。</t>
+          <t>Precision agriculture sensors, GPS guidance components, spray nozzles, pump systems, and lightweight composite materials for drone-based crop sprayers.</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>寻找价格有竞争力、能提供灵活付款条件（如延期信用证）、并支持快速交付的中国工程机械品牌及OEM供应商。</t>
+          <t>Chinese tech companies offering IoT-enabled agricultural sensors, electric motors, and battery systems with proven field performance in tropical climates.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>土耳其、卡塔尔、科威特、阿尔及利亚、莫桑比克</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>暂无</t>
+          <t>Brazil, Latin America, Africa</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Jacto has a commercial office in Shanghai for sourcing electronic components and has partnered with Chinese drone maker XAG for pilot projects.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Renaissance Construction、Enka Insaat、TAV Airports</t>
+          <t>John Deere Brazil, CNH Industrial, Stara</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>土耳其建筑市场份额约5%，在非洲机场建设领域排名前三。</t>
+          <t>~25% of Brazil's sprayer market</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>2025年中标伊拉克新港口项目，计划采购大批量工程机械。</t>
+          <t>In 2025, Jacto launched a fully autonomous electric sprayer and announced a $50 million factory expansion in Minas Gerais, with Chinese battery supplier as a key partner.</t>
         </is>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Large farm equipment manufacturer / Rental</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Enterprise (&gt;1000)</t>
+          <t>Large enterprise</t>
         </is>
       </c>
       <c r="R19" s="4" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>Major Turkish contractor with international projects, has used Chinese equipment in Africa and Middle East.</t>
+          <t>Modernizing fleet with smart agri-tech; Chinese sensors and batteries are cost-effective and align with their automation roadmap.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Arabtec Holding PJSC</t>
+          <t>Construtora Norberto Odebrecht (Novonor)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>https://www.arabtecholding.com</t>
+          <t>https://www.novonor.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>1944</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>迪拜，阿联酋</t>
+          <t>圣保罗，巴西</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>约20,000人（重组后）</t>
+          <t>约30,000人（重组后）</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>约15亿美元（2024年）</t>
+          <t>约50亿美元（2024年恢复）</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>阿联酋领先建筑承包商，专注于高层建筑、商业综合体、石油天然气设施和基础设施项目，曾参与迪拜哈利法塔建设。</t>
+          <t>巴西最大建筑公司之一，专注于大型基础设施（水坝、港口、高速公路）、能源和石油化工项目，现以Novonor品牌运营。</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>需要采购塔式起重机、施工升降机、混凝土设备、小型挖掘机，以及用于中东农业项目的灌溉和耕作机械。</t>
+          <t>需要采购土方机械（挖掘机、自卸卡车）、桩工机械、混凝土设备，以及用于农业项目的拖拉机等农业机械。</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供快速交付、适应高温环境（50°C）的中国设备商，支持海湾合作委员会（GCC）项目，并愿意合作建立区域服务中心。</t>
+          <t>寻找能提供融资支持、适应拉美工况（高海拔、湿热）的中国设备制造商，并愿意共同开发巴西市场。</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特、卡塔尔、埃及、伊拉克</t>
+          <t>巴西、拉丁美洲（秘鲁、哥伦比亚）、安哥拉、莫桑比克</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>暂无正式分公司，但通过迪拜贸易商采购中国设备</t>
+          <t>暂无正式分公司，但通过贸易商采购中国设备</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>ALEC Engineering、Dutco Construction、Six Construct (BESIX)</t>
+          <t>Andrade Gutierrez、Camargo Corrêa、Queiroz Galvão</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>阿联酋建筑市场份额约5%，重组后聚焦高端项目</t>
+          <t>巴西大型基建市场份额约7%，重组后逐步恢复</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>2025年获得阿布扎比多个住宅项目合同，计划更新机械车队。</t>
+          <t>2025年完成债务重组，重启巴西东北部灌溉工程，计划采购新机械。</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
@@ -2383,83 +2383,83 @@
         </is>
       </c>
       <c r="R20" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>Prominent UAE contractor with regional projects, known to lease and buy Chinese equipment for cost efficiency.</t>
+          <t>Major Brazilian contractor with large infrastructure and industrial projects, cost-driven and has imported Chinese machinery.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Coteccons Construction Joint Stock Company</t>
+          <t>Julius Berger Nigeria Plc</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>https://www.coteccons.vn</t>
+          <t>https://www.julius-berger.com</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>1965</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>胡志明市，越南</t>
+          <t>阿布贾，尼日利亚</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>8000</t>
+          <t>18000</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>约12亿美元</t>
+          <t>约20亿美元</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>越南最大的建筑承包商，专注于高层建筑、工业厂房和基础设施项目，同时提供建筑机械租赁服务。</t>
+          <t>尼日利亚最大的建筑和工程公司，承接道路、桥梁、港口及大型基础设施项目，同时销售建筑设备和材料。</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>需要采购塔式起重机、施工升降机、混凝土搅拌站、钢筋加工设备及小型挖掘机。</t>
+          <t>需要采购土方机械（挖掘机、推土机）、混凝土设备、起重机械及重型卡车，用于大型基建项目。</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>希望与能提供融资支持、且适应东南亚热带气候的工程机械中国厂商合作。</t>
+          <t>寻找能提供高性价比工程机械、具备非洲市场售后服务和配件供应能力的中国制造商。</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>越南、柬埔寨、老挝、缅甸</t>
+          <t>尼日利亚、西非其他国家（加纳、喀麦隆）、中非部分地区</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>暂无，但已与多家中国设备商建立直销关系。</t>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Hoa Binh Construction Group, Ricons Construction, Unicons</t>
+          <t>Dangote Group, Reynolds Construction Company, Setraco Nigeria</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>在越南高端建筑承包市场占有率约20%，排名第一。</t>
+          <t>在尼日利亚大型基建承包市场占有率约15%-20%，为行业龙头。</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布与日本合资开发越南绿色建筑项目，并计划采购电动工程机械以符合环保要求。</t>
+          <t>2025年宣布中标尼日利亚联邦政府价值8亿美元的公路升级项目，并计划采购一批新型环保工程设备。</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2469,7 +2469,7 @@
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
@@ -2478,93 +2478,93 @@
         </is>
       </c>
       <c r="R21" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>Vietnam's largest construction company, with high-rise and industrial projects, increasingly using Chinese equipment.</t>
+          <t>Leading Nigerian construction firm, heavily involved in infrastructure, has used Chinese excavators and loaders.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Al Jaber Group</t>
+          <t>Maaden (Saudi Arabian Mining Company)</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>https://www.aljabergroup.com</t>
+          <t>https://www.maaden.com.sa</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1970</t>
+          <t>1997</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>阿布扎比，阿联酋</t>
+          <t>利雅得，沙特阿拉伯</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>15000</t>
+          <t>9000</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>约35亿美元</t>
+          <t>约90亿美元</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>阿联酋多元化建筑与工程集团，业务涵盖建筑承包、重型设备租赁、物流和能源服务。</t>
+          <t>沙特国有矿业公司，主营磷酸盐、铝、黄金及基础金属开采与加工。</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>需要采购挖掘机、起重机、混凝土泵车、推土机及农业整地机械。</t>
+          <t>需要采购大型露天采矿设备、物料搬运机械、农业灌溉设备（用于矿区生态恢复）。</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>需要能提供融资支持、快速交付及海湾地区配件仓储的中国大型设备制造商。</t>
+          <t>寻找能适应沙漠高温环境、提供快速本地化服务（在沙特设点）的中国供应商。</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>阿联酋、沙特、卡塔尔、伊拉克、埃及</t>
+          <t>沙特、阿联酋、埃及、印度、中国</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>在迪拜设有采购中心，与三一重工、柳工有长期合作。</t>
+          <t>在深圳设有联合采购办公室，与中联重科有设备采购协议。</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Arabtec、ASGC、Nabco Group</t>
+          <t>沙特基础工业公司（SABIC）、阿联酋环球铝业、巴里克黄金</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>阿联酋建筑承包市场份额约10%，设备租赁市场占有率前五。</t>
+          <t>沙特矿业领域市场份额超50%，中东最大矿业公司。</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>2026年初获得阿布扎比新城基建项目，宣布采购价值8000万美元的中国工程机械。</t>
+          <t>2025年与宝武集团签署协议，采购20台大型矿用挖掘机用于新磷酸盐矿项目。</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>Construction companies &amp; contractors</t>
+          <t>Mining companies</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>UAE</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
@@ -2573,93 +2573,93 @@
         </is>
       </c>
       <c r="R22" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>Diversified UAE contractor with construction and oilfield services, has purchased Chinese cranes and loaders.</t>
+          <t>State-controlled mining company, expanding operations, price-sensitive and has used Chinese machinery in remote sites.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Petrobras</t>
+          <t>Limak Holding</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>https://www.petrobras.com.br</t>
+          <t>https://www.limak.com.tr</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1953</t>
+          <t>1976</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>里约热内卢，巴西</t>
+          <t>安卡拉，土耳其</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>45000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>约900亿美元</t>
+          <t>约60亿美元</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>巴西国家石油公司，全球深海石油开采技术领先者，业务涵盖勘探、炼化、天然气及生物燃料，拥有大量海上平台和陆上油田。</t>
+          <t>土耳其多元化集团，业务涵盖建筑、能源、水泥、港口运营和机场建设，是中东及非洲大型基建项目的总承包商。</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>需要采购石油专用工程机械（如防爆叉车、特种起重机）、管道铺设设备、油田用发电机组以及农业燃料生产所需的农机设备。</t>
+          <t>需要采购大型土方机械（挖掘机、推土机）、混凝土设备、起重机以及用于农业灌溉和土地整理的中型拖拉机。</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>寻找通过API或ISO认证、能提供耐腐蚀和防爆等级设备、并支持本地组装的中国重工企业。</t>
+          <t>寻找价格有竞争力、能提供灵活付款条件（如延期信用证）、并支持快速交付的中国工程机械品牌及OEM供应商。</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>巴西、美国、阿根廷、尼日利亚、安哥拉</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>北京设有代表处</t>
+          <t>土耳其、卡塔尔、科威特、阿尔及利亚、莫桑比克</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>暂无</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Ecopetrol、PDVSA、YPF</t>
+          <t>Renaissance Construction、Enka Insaat、TAV Airports</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>巴西石油产量市场份额约70%，深海油田技术全球领先。</t>
+          <t>土耳其建筑市场份额约5%，在非洲机场建设领域排名前三。</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布未来五年投资1000亿美元用于炼化升级，部分设备将面向亚洲采购。</t>
+          <t>2025年中标伊拉克新港口项目，计划采购大批量工程机械。</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Oil &amp; gas field service companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
@@ -2668,93 +2668,93 @@
         </is>
       </c>
       <c r="R23" s="4" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>Brazilian oil giant, uses heavy equipment for onshore and offshore operations, has tested Chinese cranes.</t>
+          <t>Major Turkish contractor with international projects, has used Chinese equipment in Africa and Middle East.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>PJSC Kamaz</t>
+          <t>Arabtec Holding PJSC</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>https://www.kamaz.ru</t>
+          <t>https://www.arabtecholding.com</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1969</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>切尔内（卡马河畔切尔内），俄罗斯</t>
+          <t>迪拜，阿联酋</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>32000</t>
+          <t>约20,000人（重组后）</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>约35亿美元</t>
+          <t>约15亿美元（2024年）</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>俄罗斯最大的卡车和重型车辆制造商，生产自卸车、牵引车、军用车辆及农用底盘，同时提供车辆维修服务。</t>
+          <t>阿联酋领先建筑承包商，专注于高层建筑、商业综合体、石油天然气设施和基础设施项目，曾参与迪拜哈利法塔建设。</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>需要采购发动机零部件、液压系统、车桥组件、电子控制系统以及农业机械配套的悬挂和传动部件。</t>
+          <t>需要采购塔式起重机、施工升降机、混凝土设备、小型挖掘机，以及用于中东农业项目的灌溉和耕作机械。</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>希望与具备IATF16949认证、能稳定供应高精度零部件的中国汽车零部件供应商建立长期合作。</t>
+          <t>寻找能提供快速交付、适应高温环境（50°C）的中国设备商，支持海湾合作委员会（GCC）项目，并愿意合作建立区域服务中心。</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>俄罗斯、独联体国家（哈萨克斯坦、白俄罗斯）、东欧、中东</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>在华设有采购代表处（上海），负责零部件采购和质量监控。</t>
+          <t>阿联酋、沙特、卡塔尔、埃及、伊拉克</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>暂无正式分公司，但通过迪拜贸易商采购中国设备</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>GAZ Group, Volvo Trucks, Daimler Truck</t>
+          <t>ALEC Engineering、Dutco Construction、Six Construct (BESIX)</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>在俄罗斯重卡市场占有率约45%，是绝对市场领导者。</t>
+          <t>阿联酋建筑市场份额约5%，重组后聚焦高端项目</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>2025年推出新一代K5系列电动卡车，并宣布与中国电池企业合作开发商用车电动化平台。</t>
+          <t>2025年获得阿布扎比多个住宅项目合同，计划更新机械车队。</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Heavy equipment distributors/dealers</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>UAE</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
@@ -2762,89 +2762,89 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R24" s="5" t="n">
-        <v>65</v>
+      <c r="R24" s="4" t="n">
+        <v>70</v>
       </c>
       <c r="S24" s="2" t="inlineStr">
         <is>
-          <t>Russian truck and machinery manufacturer, also distributes construction equipment, including Chinese brands.</t>
+          <t>Prominent UAE contractor with regional projects, known to lease and buy Chinese equipment for cost efficiency.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Hoa Phat Group</t>
+          <t>Coteccons Construction Joint Stock Company</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>https://www.hoaphat.com.vn</t>
+          <t>https://www.coteccons.vn</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>河内，越南</t>
+          <t>胡志明市，越南</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>8000</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>约80亿美元</t>
+          <t>约12亿美元</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>越南最大钢铁生产商，同时涉足建筑、房地产和农业机械制造，其农机品牌在东南亚市场具有较高知名度。</t>
+          <t>越南最大的建筑承包商，专注于高层建筑、工业厂房和基础设施项目，同时提供建筑机械租赁服务。</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>需要采购钢材加工设备、大型铸造机械、农业机械核心部件（如发动机、变速箱）以及自动化焊接机器人。</t>
+          <t>需要采购塔式起重机、施工升降机、混凝土搅拌站、钢筋加工设备及小型挖掘机。</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>寻找能提供技术转让、共同开发适合东南亚水稻种植的小型农机的中国制造商，以及钢铁冶炼设备供应商。</t>
+          <t>希望与能提供融资支持、且适应东南亚热带气候的工程机械中国厂商合作。</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>越南、柬埔寨、老挝、缅甸、泰国</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>在广西南宁设有贸易办事处</t>
+          <t>越南、柬埔寨、老挝、缅甸</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>暂无，但已与多家中国设备商建立直销关系。</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Formosa Ha Tinh、Tata Steel、SMC</t>
+          <t>Hoa Binh Construction Group, Ricons Construction, Unicons</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>越南建筑钢材市场份额约30%，农机市场份额约15%。</t>
+          <t>在越南高端建筑承包市场占有率约20%，排名第一。</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>2025年宣布投资建设新农机装配厂，计划从中国引进两条智能生产线。</t>
+          <t>2025年宣布与日本合资开发越南绿色建筑项目，并计划采购电动工程机械以符合环保要求。</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>Mining companies</t>
+          <t>Construction companies &amp; contractors</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2857,112 +2857,492 @@
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R25" s="5" t="n">
-        <v>65</v>
+      <c r="R25" s="4" t="n">
+        <v>70</v>
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>Vietnam's largest steel producer, with mining and construction divisions, has imported Chinese heavy machinery.</t>
+          <t>Vietnam's largest construction company, with high-rise and industrial projects, increasingly using Chinese equipment.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Al Jaber Group</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.aljabergroup.com</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>阿布扎比，阿联酋</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>约35亿美元</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋多元化建筑与工程集团，业务涵盖建筑承包、重型设备租赁、物流和能源服务。</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>需要采购挖掘机、起重机、混凝土泵车、推土机及农业整地机械。</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>需要能提供融资支持、快速交付及海湾地区配件仓储的中国大型设备制造商。</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋、沙特、卡塔尔、伊拉克、埃及</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>在迪拜设有采购中心，与三一重工、柳工有长期合作。</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Arabtec、ASGC、Nabco Group</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>阿联酋建筑承包市场份额约10%，设备租赁市场占有率前五。</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>2026年初获得阿布扎比新城基建项目，宣布采购价值8000万美元的中国工程机械。</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Construction companies &amp; contractors</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R26" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>Diversified UAE contractor with construction and oilfield services, has purchased Chinese cranes and loaders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Petrobras</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.petrobras.com.br</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>1953</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>里约热内卢，巴西</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>45000</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>约900亿美元</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>巴西国家石油公司，全球深海石油开采技术领先者，业务涵盖勘探、炼化、天然气及生物燃料，拥有大量海上平台和陆上油田。</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>需要采购石油专用工程机械（如防爆叉车、特种起重机）、管道铺设设备、油田用发电机组以及农业燃料生产所需的农机设备。</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>寻找通过API或ISO认证、能提供耐腐蚀和防爆等级设备、并支持本地组装的中国重工企业。</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>巴西、美国、阿根廷、尼日利亚、安哥拉</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>北京设有代表处</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Ecopetrol、PDVSA、YPF</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>巴西石油产量市场份额约70%，深海油田技术全球领先。</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布未来五年投资1000亿美元用于炼化升级，部分设备将面向亚洲采购。</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>Oil &amp; gas field service companies</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R27" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>Brazilian oil giant, uses heavy equipment for onshore and offshore operations, has tested Chinese cranes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>PJSC Kamaz</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kamaz.ru</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>1969</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>切尔内（卡马河畔切尔内），俄罗斯</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>32000</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>约35亿美元</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>俄罗斯最大的卡车和重型车辆制造商，生产自卸车、牵引车、军用车辆及农用底盘，同时提供车辆维修服务。</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>需要采购发动机零部件、液压系统、车桥组件、电子控制系统以及农业机械配套的悬挂和传动部件。</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>希望与具备IATF16949认证、能稳定供应高精度零部件的中国汽车零部件供应商建立长期合作。</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>俄罗斯、独联体国家（哈萨克斯坦、白俄罗斯）、东欧、中东</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>在华设有采购代表处（上海），负责零部件采购和质量监控。</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>GAZ Group, Volvo Trucks, Daimler Truck</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>在俄罗斯重卡市场占有率约45%，是绝对市场领导者。</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>2025年推出新一代K5系列电动卡车，并宣布与中国电池企业合作开发商用车电动化平台。</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Heavy equipment distributors/dealers</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>Russian truck and machinery manufacturer, also distributes construction equipment, including Chinese brands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Hoa Phat Group</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hoaphat.com.vn</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>河内，越南</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>约80亿美元</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>越南最大钢铁生产商，同时涉足建筑、房地产和农业机械制造，其农机品牌在东南亚市场具有较高知名度。</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>需要采购钢材加工设备、大型铸造机械、农业机械核心部件（如发动机、变速箱）以及自动化焊接机器人。</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>寻找能提供技术转让、共同开发适合东南亚水稻种植的小型农机的中国制造商，以及钢铁冶炼设备供应商。</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>越南、柬埔寨、老挝、缅甸、泰国</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>在广西南宁设有贸易办事处</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Formosa Ha Tinh、Tata Steel、SMC</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>越南建筑钢材市场份额约30%，农机市场份额约15%。</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>2025年宣布投资建设新农机装配厂，计划从中国引进两条智能生产线。</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>Mining companies</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise (&gt;1000)</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam's largest steel producer, with mining and construction divisions, has imported Chinese heavy machinery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Rostec State Corporation</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>https://rostec.ru</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>莫斯科，俄罗斯</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>450000</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>约280亿美元</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>俄罗斯国有军工及工业集团，涵盖航空、电子、武器、汽车、医疗设备等多元领域，旗下拥有多家工程机械和特种车辆制造企业。</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>需要从中国采购液压元件、发动机零部件、工程机械整机（如挖掘机、装载机）以及农业机械（如拖拉机、收割机）的替代零部件和生产线设备。</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>寻找具备军工或重工配套资质、能适应俄罗斯极端气候、提供本地化售后服务的中国大型制造企业或系统集成商。</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>俄罗斯、印度、中东、非洲、东南亚</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>北京设有代表处</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Uralvagonzavod、Almaz-Antey、Sukhoi</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>俄罗斯军工出口份额约50%，国内工业制造领域占据主导地位。</t>
         </is>
       </c>
-      <c r="N26" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>2025年计划扩大民用工程机械产能，并寻求与中国在无人机和特种车辆领域的联合开发。</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr">
         <is>
           <t>Government infrastructure procurement</t>
         </is>
       </c>
-      <c r="P26" s="2" t="inlineStr">
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>Russia</t>
         </is>
       </c>
-      <c r="Q26" s="2" t="inlineStr">
+      <c r="Q30" s="2" t="inlineStr">
         <is>
           <t>Enterprise (&gt;1000)</t>
         </is>
       </c>
-      <c r="R26" s="5" t="n">
+      <c r="R30" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="S26" s="2" t="inlineStr">
+      <c r="S30" s="2" t="inlineStr">
         <is>
           <t>Russian state conglomerate, indirectly procures heavy equipment for infrastructure, has partnered with Chinese firms.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S26"/>
+  <autoFilter ref="A1:S30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>